<commit_message>
Expose the getNrOfDihedralAngles method
</commit_message>
<xml_diff>
--- a/src/pylimer_tools/data/everaers_et_al_unit_properties.xlsx
+++ b/src/pylimer_tools/data/everaers_et_al_unit_properties.xlsx
@@ -16,7 +16,7 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="61" uniqueCount="61">
   <si>
-    <t>name</t>
+    <t>zot</t>
   </si>
   <si>
     <t>T_ref</t>
@@ -204,7 +204,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" mc:Ignorable="x14ac">
   <numFmts count="0"/>
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -215,6 +215,12 @@
     <font>
       <sz val="11"/>
       <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
       <name val="Calibri"/>
       <family val="2"/>
     </font>
@@ -251,16 +257,16 @@
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
       <alignment horizontal="general"/>
     </xf>
-    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf xfId="0" numFmtId="4" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
     <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
     <xf xfId="0" numFmtId="4" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf xfId="0" numFmtId="4" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
@@ -673,7 +679,7 @@
         <v>22</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="18">
+    <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="19.5">
       <c r="A2" s="1" t="s">
         <v>23</v>
       </c>
@@ -744,7 +750,7 @@
         <v>32</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="18">
+    <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="19.5">
       <c r="A3" s="1" t="s">
         <v>24</v>
       </c>
@@ -815,7 +821,7 @@
         <v>41.3</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="18">
+    <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="19.5">
       <c r="A4" s="1" t="s">
         <v>25</v>
       </c>
@@ -886,7 +892,7 @@
         <v>17.6</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="18">
+    <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="19.5">
       <c r="A5" s="1" t="s">
         <v>26</v>
       </c>
@@ -957,7 +963,7 @@
         <v>37.1</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="6" customHeight="1" ht="18">
+    <row x14ac:dyDescent="0.25" r="6" customHeight="1" ht="19.5">
       <c r="A6" s="1" t="s">
         <v>27</v>
       </c>
@@ -1028,7 +1034,7 @@
         <v>33.1</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="7" customHeight="1" ht="18">
+    <row x14ac:dyDescent="0.25" r="7" customHeight="1" ht="19.5">
       <c r="A7" s="1" t="s">
         <v>28</v>
       </c>
@@ -1099,7 +1105,7 @@
         <v>61.3</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="8" customHeight="1" ht="18">
+    <row x14ac:dyDescent="0.25" r="8" customHeight="1" ht="19.5">
       <c r="A8" s="1" t="s">
         <v>29</v>
       </c>
@@ -1170,7 +1176,7 @@
         <v>27.3</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="9" customHeight="1" ht="18">
+    <row x14ac:dyDescent="0.25" r="9" customHeight="1" ht="19.5">
       <c r="A9" s="1" t="s">
         <v>30</v>
       </c>
@@ -1241,7 +1247,7 @@
         <v>44</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="10" customHeight="1" ht="18">
+    <row x14ac:dyDescent="0.25" r="10" customHeight="1" ht="19.5">
       <c r="A10" s="1" t="s">
         <v>31</v>
       </c>
@@ -1312,7 +1318,7 @@
         <v>40.7</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="11" customHeight="1" ht="18">
+    <row x14ac:dyDescent="0.25" r="11" customHeight="1" ht="19.5">
       <c r="A11" s="1" t="s">
         <v>32</v>
       </c>
@@ -1383,7 +1389,7 @@
         <v>40.4</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="12" customHeight="1" ht="18">
+    <row x14ac:dyDescent="0.25" r="12" customHeight="1" ht="19.5">
       <c r="A12" s="1" t="s">
         <v>33</v>
       </c>
@@ -1454,7 +1460,7 @@
         <v>38.2</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="13" customHeight="1" ht="18">
+    <row x14ac:dyDescent="0.25" r="13" customHeight="1" ht="19.5">
       <c r="A13" s="1" t="s">
         <v>34</v>
       </c>
@@ -1525,7 +1531,7 @@
         <v>34.3</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="14" customHeight="1" ht="18">
+    <row x14ac:dyDescent="0.25" r="14" customHeight="1" ht="19.5">
       <c r="A14" s="1" t="s">
         <v>35</v>
       </c>
@@ -1596,7 +1602,7 @@
         <v>30.7</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="15" customHeight="1" ht="18">
+    <row x14ac:dyDescent="0.25" r="15" customHeight="1" ht="19.5">
       <c r="A15" s="1" t="s">
         <v>36</v>
       </c>
@@ -1667,7 +1673,7 @@
         <v>22.2</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="16" customHeight="1" ht="18">
+    <row x14ac:dyDescent="0.25" r="16" customHeight="1" ht="19.5">
       <c r="A16" s="1" t="s">
         <v>37</v>
       </c>
@@ -1738,7 +1744,7 @@
         <v>17.6</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="17" customHeight="1" ht="18">
+    <row x14ac:dyDescent="0.25" r="17" customHeight="1" ht="19.5">
       <c r="A17" s="1" t="s">
         <v>38</v>
       </c>
@@ -1809,7 +1815,7 @@
         <v>13.2</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="18" customHeight="1" ht="18">
+    <row x14ac:dyDescent="0.25" r="18" customHeight="1" ht="19.5">
       <c r="A18" s="1" t="s">
         <v>39</v>
       </c>
@@ -1880,7 +1886,7 @@
         <v>15.6</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="19" customHeight="1" ht="18">
+    <row x14ac:dyDescent="0.25" r="19" customHeight="1" ht="19.5">
       <c r="A19" s="1" t="s">
         <v>40</v>
       </c>
@@ -1951,7 +1957,7 @@
         <v>15.9</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="20" customHeight="1" ht="18">
+    <row x14ac:dyDescent="0.25" r="20" customHeight="1" ht="19.5">
       <c r="A20" s="1" t="s">
         <v>41</v>
       </c>
@@ -2022,7 +2028,7 @@
         <v>52.2</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="21" customHeight="1" ht="18">
+    <row x14ac:dyDescent="0.25" r="21" customHeight="1" ht="19.5">
       <c r="A21" s="1" t="s">
         <v>42</v>
       </c>
@@ -2093,7 +2099,7 @@
         <v>13.2</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="22" customHeight="1" ht="18">
+    <row x14ac:dyDescent="0.25" r="22" customHeight="1" ht="19.5">
       <c r="A22" s="1" t="s">
         <v>43</v>
       </c>
@@ -2164,7 +2170,7 @@
         <v>23.1</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="23" customHeight="1" ht="18">
+    <row x14ac:dyDescent="0.25" r="23" customHeight="1" ht="19.5">
       <c r="A23" s="1" t="s">
         <v>44</v>
       </c>
@@ -2235,7 +2241,7 @@
         <v>80.2</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="24" customHeight="1" ht="18">
+    <row x14ac:dyDescent="0.25" r="24" customHeight="1" ht="19.5">
       <c r="A24" s="1" t="s">
         <v>46</v>
       </c>
@@ -2306,7 +2312,7 @@
         <v>111.5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="25" customHeight="1" ht="18">
+    <row x14ac:dyDescent="0.25" r="25" customHeight="1" ht="19.5">
       <c r="A25" s="1" t="s">
         <v>47</v>
       </c>
@@ -2377,7 +2383,7 @@
         <v>5.7</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="26" customHeight="1" ht="18">
+    <row x14ac:dyDescent="0.25" r="26" customHeight="1" ht="19.5">
       <c r="A26" s="1" t="s">
         <v>48</v>
       </c>
@@ -2448,7 +2454,7 @@
         <v>16.7</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="27" customHeight="1" ht="18">
+    <row x14ac:dyDescent="0.25" r="27" customHeight="1" ht="19.5">
       <c r="A27" s="1" t="s">
         <v>50</v>
       </c>
@@ -2519,7 +2525,7 @@
         <v>40.6</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="28" customHeight="1" ht="18">
+    <row x14ac:dyDescent="0.25" r="28" customHeight="1" ht="19.5">
       <c r="A28" s="1" t="s">
         <v>51</v>
       </c>
@@ -2590,7 +2596,7 @@
         <v>100.9</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="29" customHeight="1" ht="18">
+    <row x14ac:dyDescent="0.25" r="29" customHeight="1" ht="19.5">
       <c r="A29" s="1" t="s">
         <v>52</v>
       </c>
@@ -2661,7 +2667,7 @@
         <v>13.9</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="30" customHeight="1" ht="18">
+    <row x14ac:dyDescent="0.25" r="30" customHeight="1" ht="19.5">
       <c r="A30" s="1" t="s">
         <v>53</v>
       </c>
@@ -2732,7 +2738,7 @@
         <v>12.8</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="31" customHeight="1" ht="18">
+    <row x14ac:dyDescent="0.25" r="31" customHeight="1" ht="19.5">
       <c r="A31" s="1" t="s">
         <v>54</v>
       </c>
@@ -2803,7 +2809,7 @@
         <v>63.4</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="32" customHeight="1" ht="18">
+    <row x14ac:dyDescent="0.25" r="32" customHeight="1" ht="19.5">
       <c r="A32" s="1" t="s">
         <v>55</v>
       </c>
@@ -2874,7 +2880,7 @@
         <v>40.5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="33" customHeight="1" ht="18">
+    <row x14ac:dyDescent="0.25" r="33" customHeight="1" ht="19.5">
       <c r="A33" s="1" t="s">
         <v>56</v>
       </c>
@@ -2945,7 +2951,7 @@
         <v>69</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="34" customHeight="1" ht="18">
+    <row x14ac:dyDescent="0.25" r="34" customHeight="1" ht="19.5">
       <c r="A34" s="1" t="s">
         <v>57</v>
       </c>

</xml_diff>

<commit_message>
Implement new method to compute soluble weight fraction from MEHP
</commit_message>
<xml_diff>
--- a/src/pylimer_tools/data/everaers_et_al_unit_properties.xlsx
+++ b/src/pylimer_tools/data/everaers_et_al_unit_properties.xlsx
@@ -16,7 +16,7 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="61" uniqueCount="61">
   <si>
-    <t>zot</t>
+    <t>name</t>
   </si>
   <si>
     <t>T_ref</t>
@@ -204,19 +204,13 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" mc:Ignorable="x14ac">
   <numFmts count="0"/>
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
     </font>
     <font>
       <sz val="11"/>
@@ -252,7 +246,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="7">
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0"/>
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
       <alignment horizontal="general"/>
@@ -261,12 +255,6 @@
       <alignment horizontal="right"/>
     </xf>
     <xf xfId="0" numFmtId="4" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf xfId="0" numFmtId="4" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
@@ -583,32 +571,32 @@
   <dimension ref="A1:W37"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" style="6" width="13.005" customWidth="1" bestFit="1"/>
-    <col min="2" max="2" style="7" width="13.005" customWidth="1" bestFit="1"/>
-    <col min="3" max="3" style="8" width="13.005" customWidth="1" bestFit="1"/>
-    <col min="4" max="4" style="8" width="13.005" customWidth="1" bestFit="1"/>
-    <col min="5" max="5" style="8" width="13.005" customWidth="1" bestFit="1"/>
-    <col min="6" max="6" style="8" width="13.005" customWidth="1" bestFit="1"/>
-    <col min="7" max="7" style="8" width="13.005" customWidth="1" bestFit="1"/>
-    <col min="8" max="8" style="8" width="13.005" customWidth="1" bestFit="1"/>
-    <col min="9" max="9" style="8" width="13.005" customWidth="1" bestFit="1"/>
-    <col min="10" max="10" style="8" width="13.005" customWidth="1" bestFit="1"/>
-    <col min="11" max="11" style="8" width="13.005" customWidth="1" bestFit="1"/>
-    <col min="12" max="12" style="8" width="13.005" customWidth="1" bestFit="1"/>
-    <col min="13" max="13" style="8" width="13.005" customWidth="1" bestFit="1"/>
-    <col min="14" max="14" style="8" width="13.005" customWidth="1" bestFit="1"/>
-    <col min="15" max="15" style="8" width="13.005" customWidth="1" bestFit="1"/>
-    <col min="16" max="16" style="8" width="13.005" customWidth="1" bestFit="1"/>
-    <col min="17" max="17" style="8" width="13.005" customWidth="1" bestFit="1"/>
-    <col min="18" max="18" style="8" width="13.005" customWidth="1" bestFit="1"/>
-    <col min="19" max="19" style="8" width="13.005" customWidth="1" bestFit="1"/>
-    <col min="20" max="20" style="8" width="13.005" customWidth="1" bestFit="1"/>
-    <col min="21" max="21" style="8" width="14.147857142857141" customWidth="1" bestFit="1"/>
-    <col min="22" max="22" style="8" width="13.005" customWidth="1" bestFit="1"/>
-    <col min="23" max="23" style="8" width="13.005" customWidth="1" bestFit="1"/>
+    <col min="1" max="1" style="4" width="13.005" customWidth="1" bestFit="1"/>
+    <col min="2" max="2" style="5" width="13.005" customWidth="1" bestFit="1"/>
+    <col min="3" max="3" style="6" width="13.005" customWidth="1" bestFit="1"/>
+    <col min="4" max="4" style="6" width="13.005" customWidth="1" bestFit="1"/>
+    <col min="5" max="5" style="6" width="13.005" customWidth="1" bestFit="1"/>
+    <col min="6" max="6" style="6" width="13.005" customWidth="1" bestFit="1"/>
+    <col min="7" max="7" style="6" width="13.005" customWidth="1" bestFit="1"/>
+    <col min="8" max="8" style="6" width="13.005" customWidth="1" bestFit="1"/>
+    <col min="9" max="9" style="6" width="13.005" customWidth="1" bestFit="1"/>
+    <col min="10" max="10" style="6" width="13.005" customWidth="1" bestFit="1"/>
+    <col min="11" max="11" style="6" width="13.005" customWidth="1" bestFit="1"/>
+    <col min="12" max="12" style="6" width="13.005" customWidth="1" bestFit="1"/>
+    <col min="13" max="13" style="6" width="13.005" customWidth="1" bestFit="1"/>
+    <col min="14" max="14" style="6" width="13.005" customWidth="1" bestFit="1"/>
+    <col min="15" max="15" style="6" width="13.005" customWidth="1" bestFit="1"/>
+    <col min="16" max="16" style="6" width="13.005" customWidth="1" bestFit="1"/>
+    <col min="17" max="17" style="6" width="13.005" customWidth="1" bestFit="1"/>
+    <col min="18" max="18" style="6" width="13.005" customWidth="1" bestFit="1"/>
+    <col min="19" max="19" style="6" width="13.005" customWidth="1" bestFit="1"/>
+    <col min="20" max="20" style="6" width="13.005" customWidth="1" bestFit="1"/>
+    <col min="21" max="21" style="6" width="14.147857142857141" customWidth="1" bestFit="1"/>
+    <col min="22" max="22" style="6" width="13.005" customWidth="1" bestFit="1"/>
+    <col min="23" max="23" style="6" width="13.005" customWidth="1" bestFit="1"/>
   </cols>
   <sheetData>
-    <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="18">
+    <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="19.5">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -683,70 +671,70 @@
       <c r="A2" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="B2" s="4">
+      <c r="B2" s="2">
         <v>298</v>
       </c>
-      <c r="C2" s="5">
+      <c r="C2" s="3">
         <v>0.528</v>
       </c>
-      <c r="D2" s="5">
+      <c r="D2" s="3">
         <v>0.893</v>
       </c>
-      <c r="E2" s="5">
+      <c r="E2" s="3">
         <v>0.51</v>
       </c>
-      <c r="F2" s="5">
+      <c r="F2" s="3">
         <v>3.52</v>
       </c>
-      <c r="G2" s="5">
+      <c r="G2" s="3">
         <v>47.7</v>
       </c>
-      <c r="H2" s="5">
+      <c r="H2" s="3">
         <v>2.5</v>
       </c>
-      <c r="I2" s="5">
+      <c r="I2" s="3">
         <v>8.8</v>
       </c>
-      <c r="J2" s="5">
+      <c r="J2" s="3">
         <v>146.6</v>
       </c>
-      <c r="K2" s="5">
+      <c r="K2" s="3">
         <v>2.15</v>
       </c>
-      <c r="L2" s="5">
+      <c r="L2" s="3">
         <v>3.66</v>
       </c>
-      <c r="M2" s="5">
+      <c r="M2" s="3">
         <v>0.085</v>
       </c>
-      <c r="N2" s="5">
+      <c r="N2" s="3">
         <v>29.41</v>
       </c>
-      <c r="O2" s="5">
+      <c r="O2" s="3">
         <v>13.6</v>
       </c>
-      <c r="P2" s="5">
+      <c r="P2" s="3">
         <v>-0.378</v>
       </c>
-      <c r="Q2" s="5">
+      <c r="Q2" s="3">
         <v>1.81</v>
       </c>
-      <c r="R2" s="5">
+      <c r="R2" s="3">
         <v>1.74</v>
       </c>
-      <c r="S2" s="5">
+      <c r="S2" s="3">
         <v>0.84</v>
       </c>
-      <c r="T2" s="5">
+      <c r="T2" s="3">
         <v>81.13</v>
       </c>
-      <c r="U2" s="5">
+      <c r="U2" s="3">
         <v>4.11</v>
       </c>
-      <c r="V2" s="5">
+      <c r="V2" s="3">
         <v>0.5</v>
       </c>
-      <c r="W2" s="4">
+      <c r="W2" s="2">
         <v>32</v>
       </c>
     </row>
@@ -754,70 +742,70 @@
       <c r="A3" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="B3" s="4">
+      <c r="B3" s="2">
         <v>298</v>
       </c>
-      <c r="C3" s="5">
+      <c r="C3" s="3">
         <v>0.596</v>
       </c>
-      <c r="D3" s="5">
+      <c r="D3" s="3">
         <v>0.9</v>
       </c>
-      <c r="E3" s="5">
+      <c r="E3" s="3">
         <v>0.44</v>
       </c>
-      <c r="F3" s="5">
+      <c r="F3" s="3">
         <v>3.1</v>
       </c>
-      <c r="G3" s="5">
+      <c r="G3" s="3">
         <v>55.1</v>
       </c>
-      <c r="H3" s="5">
+      <c r="H3" s="3">
         <v>2.72</v>
       </c>
-      <c r="I3" s="5">
+      <c r="I3" s="3">
         <v>8.44</v>
       </c>
-      <c r="J3" s="5">
+      <c r="J3" s="3">
         <v>119.6</v>
       </c>
-      <c r="K3" s="5">
+      <c r="K3" s="3">
         <v>1.76</v>
       </c>
-      <c r="L3" s="5">
+      <c r="L3" s="3">
         <v>4.52</v>
       </c>
-      <c r="M3" s="5">
+      <c r="M3" s="3">
         <v>0.064</v>
       </c>
-      <c r="N3" s="5">
+      <c r="N3" s="3">
         <v>42.55</v>
       </c>
-      <c r="O3" s="5">
+      <c r="O3" s="3">
         <v>17.8</v>
       </c>
-      <c r="P3" s="5">
+      <c r="P3" s="3">
         <v>-0.086</v>
       </c>
-      <c r="Q3" s="5">
+      <c r="Q3" s="3">
         <v>1.89</v>
       </c>
-      <c r="R3" s="5">
+      <c r="R3" s="3">
         <v>1.82</v>
       </c>
-      <c r="S3" s="5">
+      <c r="S3" s="3">
         <v>1.07</v>
       </c>
-      <c r="T3" s="5">
+      <c r="T3" s="3">
         <v>63.37</v>
       </c>
-      <c r="U3" s="5">
+      <c r="U3" s="3">
         <v>4.11</v>
       </c>
-      <c r="V3" s="5">
+      <c r="V3" s="3">
         <v>0.46</v>
       </c>
-      <c r="W3" s="5">
+      <c r="W3" s="3">
         <v>41.3</v>
       </c>
     </row>
@@ -825,70 +813,70 @@
       <c r="A4" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="B4" s="4">
+      <c r="B4" s="2">
         <v>298</v>
       </c>
-      <c r="C4" s="5">
+      <c r="C4" s="3">
         <v>0.422</v>
       </c>
-      <c r="D4" s="5">
+      <c r="D4" s="3">
         <v>0.97</v>
       </c>
-      <c r="E4" s="5">
+      <c r="E4" s="3">
         <v>0.25</v>
       </c>
-      <c r="F4" s="5">
+      <c r="F4" s="3">
         <v>4.06</v>
       </c>
-      <c r="G4" s="5">
+      <c r="G4" s="3">
         <v>63.7</v>
       </c>
-      <c r="H4" s="5">
+      <c r="H4" s="3">
         <v>2.82</v>
       </c>
-      <c r="I4" s="5">
+      <c r="I4" s="3">
         <v>11.42</v>
       </c>
-      <c r="J4" s="5">
+      <c r="J4" s="3">
         <v>309.28</v>
       </c>
-      <c r="K4" s="5">
+      <c r="K4" s="3">
         <v>4.17</v>
       </c>
-      <c r="L4" s="5">
+      <c r="L4" s="3">
         <v>1.89</v>
       </c>
-      <c r="M4" s="5">
+      <c r="M4" s="3">
         <v>0.091</v>
       </c>
-      <c r="N4" s="5">
+      <c r="N4" s="3">
         <v>31.08</v>
       </c>
-      <c r="O4" s="5">
+      <c r="O4" s="3">
         <v>15.7</v>
       </c>
-      <c r="P4" s="5">
+      <c r="P4" s="3">
         <v>0.013</v>
       </c>
-      <c r="Q4" s="5">
+      <c r="Q4" s="3">
         <v>1.92</v>
       </c>
-      <c r="R4" s="5">
+      <c r="R4" s="3">
         <v>1.85</v>
       </c>
-      <c r="S4" s="5">
+      <c r="S4" s="3">
         <v>0.46</v>
       </c>
-      <c r="T4" s="5">
+      <c r="T4" s="3">
         <v>161.05</v>
       </c>
-      <c r="U4" s="5">
+      <c r="U4" s="3">
         <v>4.11</v>
       </c>
-      <c r="V4" s="5">
+      <c r="V4" s="3">
         <v>0.62</v>
       </c>
-      <c r="W4" s="5">
+      <c r="W4" s="3">
         <v>17.6</v>
       </c>
     </row>
@@ -896,70 +884,70 @@
       <c r="A5" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="B5" s="4">
+      <c r="B5" s="2">
         <v>298</v>
       </c>
-      <c r="C5" s="5">
+      <c r="C5" s="3">
         <v>0.591</v>
       </c>
-      <c r="D5" s="5">
+      <c r="D5" s="3">
         <v>0.898</v>
       </c>
-      <c r="E5" s="5">
+      <c r="E5" s="3">
         <v>0.44</v>
       </c>
-      <c r="F5" s="5">
+      <c r="F5" s="3">
         <v>3.13</v>
       </c>
-      <c r="G5" s="5">
+      <c r="G5" s="3">
         <v>54.8</v>
       </c>
-      <c r="H5" s="5">
+      <c r="H5" s="3">
         <v>2.86</v>
       </c>
-      <c r="I5" s="5">
+      <c r="I5" s="3">
         <v>8.98</v>
       </c>
-      <c r="J5" s="5">
+      <c r="J5" s="3">
         <v>136.5</v>
       </c>
-      <c r="K5" s="4">
+      <c r="K5" s="2">
         <v>2</v>
       </c>
-      <c r="L5" s="5">
+      <c r="L5" s="3">
         <v>3.95</v>
       </c>
-      <c r="M5" s="5">
+      <c r="M5" s="3">
         <v>0.077</v>
       </c>
-      <c r="N5" s="5">
+      <c r="N5" s="3">
         <v>37.17</v>
       </c>
-      <c r="O5" s="5">
+      <c r="O5" s="3">
         <v>17.5</v>
       </c>
-      <c r="P5" s="5">
+      <c r="P5" s="3">
         <v>0.056</v>
       </c>
-      <c r="Q5" s="5">
+      <c r="Q5" s="3">
         <v>1.94</v>
       </c>
-      <c r="R5" s="5">
+      <c r="R5" s="3">
         <v>1.87</v>
       </c>
-      <c r="S5" s="5">
+      <c r="S5" s="3">
         <v>0.97</v>
       </c>
-      <c r="T5" s="5">
+      <c r="T5" s="3">
         <v>70.5</v>
       </c>
-      <c r="U5" s="5">
+      <c r="U5" s="3">
         <v>4.11</v>
       </c>
-      <c r="V5" s="5">
+      <c r="V5" s="3">
         <v>0.48</v>
       </c>
-      <c r="W5" s="5">
+      <c r="W5" s="3">
         <v>37.1</v>
       </c>
     </row>
@@ -967,70 +955,70 @@
       <c r="A6" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="B6" s="4">
+      <c r="B6" s="2">
         <v>298</v>
       </c>
-      <c r="C6" s="5">
+      <c r="C6" s="3">
         <v>0.585</v>
       </c>
-      <c r="D6" s="5">
+      <c r="D6" s="3">
         <v>0.965</v>
       </c>
-      <c r="E6" s="5">
+      <c r="E6" s="3">
         <v>0.44</v>
       </c>
-      <c r="F6" s="5">
+      <c r="F6" s="3">
         <v>2.94</v>
       </c>
-      <c r="G6" s="5">
+      <c r="G6" s="3">
         <v>56.5</v>
       </c>
-      <c r="H6" s="5">
+      <c r="H6" s="3">
         <v>3.02</v>
       </c>
-      <c r="I6" s="5">
+      <c r="I6" s="3">
         <v>9.58</v>
       </c>
-      <c r="J6" s="5">
+      <c r="J6" s="3">
         <v>156.9</v>
       </c>
-      <c r="K6" s="5">
+      <c r="K6" s="3">
         <v>2.3</v>
       </c>
-      <c r="L6" s="5">
+      <c r="L6" s="3">
         <v>3.44</v>
       </c>
-      <c r="M6" s="5">
+      <c r="M6" s="3">
         <v>0.093</v>
       </c>
-      <c r="N6" s="5">
+      <c r="N6" s="3">
         <v>32.32</v>
       </c>
-      <c r="O6" s="5">
+      <c r="O6" s="3">
         <v>19.2</v>
       </c>
-      <c r="P6" s="5">
+      <c r="P6" s="3">
         <v>0.191</v>
       </c>
-      <c r="Q6" s="5">
+      <c r="Q6" s="3">
         <v>1.99</v>
       </c>
-      <c r="R6" s="5">
+      <c r="R6" s="3">
         <v>1.92</v>
       </c>
-      <c r="S6" s="5">
+      <c r="S6" s="3">
         <v>0.86</v>
       </c>
-      <c r="T6" s="5">
+      <c r="T6" s="3">
         <v>78.86</v>
       </c>
-      <c r="U6" s="5">
+      <c r="U6" s="3">
         <v>4.11</v>
       </c>
-      <c r="V6" s="5">
+      <c r="V6" s="3">
         <v>0.5</v>
       </c>
-      <c r="W6" s="5">
+      <c r="W6" s="3">
         <v>33.1</v>
       </c>
     </row>
@@ -1038,70 +1026,70 @@
       <c r="A7" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="B7" s="4">
+      <c r="B7" s="2">
         <v>298</v>
       </c>
-      <c r="C7" s="5">
+      <c r="C7" s="3">
         <v>0.758</v>
       </c>
-      <c r="D7" s="5">
+      <c r="D7" s="3">
         <v>0.9</v>
       </c>
-      <c r="E7" s="5">
+      <c r="E7" s="3">
         <v>0.95</v>
       </c>
-      <c r="F7" s="5">
+      <c r="F7" s="3">
         <v>2.43</v>
       </c>
-      <c r="G7" s="5">
+      <c r="G7" s="3">
         <v>42.2</v>
       </c>
-      <c r="H7" s="5">
+      <c r="H7" s="3">
         <v>3.4</v>
       </c>
-      <c r="I7" s="5">
+      <c r="I7" s="3">
         <v>8.28</v>
       </c>
-      <c r="J7" s="5">
+      <c r="J7" s="3">
         <v>90.5</v>
       </c>
-      <c r="K7" s="5">
+      <c r="K7" s="3">
         <v>1.67</v>
       </c>
-      <c r="L7" s="5">
+      <c r="L7" s="3">
         <v>5.99</v>
       </c>
-      <c r="M7" s="5">
+      <c r="M7" s="3">
         <v>0.131</v>
       </c>
-      <c r="N7" s="5">
+      <c r="N7" s="3">
         <v>25.93</v>
       </c>
-      <c r="O7" s="5">
+      <c r="O7" s="3">
         <v>17.3</v>
       </c>
-      <c r="P7" s="5">
+      <c r="P7" s="3">
         <v>0.445</v>
       </c>
-      <c r="Q7" s="5">
+      <c r="Q7" s="3">
         <v>2.11</v>
       </c>
-      <c r="R7" s="5">
+      <c r="R7" s="3">
         <v>2.04</v>
       </c>
-      <c r="S7" s="5">
+      <c r="S7" s="3">
         <v>1.26</v>
       </c>
-      <c r="T7" s="5">
+      <c r="T7" s="3">
         <v>42.87</v>
       </c>
-      <c r="U7" s="5">
+      <c r="U7" s="3">
         <v>4.11</v>
       </c>
-      <c r="V7" s="5">
+      <c r="V7" s="3">
         <v>0.41</v>
       </c>
-      <c r="W7" s="5">
+      <c r="W7" s="3">
         <v>61.3</v>
       </c>
     </row>
@@ -1109,70 +1097,70 @@
       <c r="A8" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="B8" s="4">
+      <c r="B8" s="2">
         <v>413</v>
       </c>
-      <c r="C8" s="5">
+      <c r="C8" s="3">
         <v>0.557</v>
       </c>
-      <c r="D8" s="5">
+      <c r="D8" s="3">
         <v>0.849</v>
       </c>
-      <c r="E8" s="5">
+      <c r="E8" s="3">
         <v>0.38</v>
       </c>
-      <c r="F8" s="5">
+      <c r="F8" s="3">
         <v>3.51</v>
       </c>
-      <c r="G8" s="5">
+      <c r="G8" s="3">
         <v>65.8</v>
       </c>
-      <c r="H8" s="5">
+      <c r="H8" s="3">
         <v>3.47</v>
       </c>
-      <c r="I8" s="5">
+      <c r="I8" s="3">
         <v>12.2</v>
       </c>
-      <c r="J8" s="5">
+      <c r="J8" s="3">
         <v>267.9</v>
       </c>
-      <c r="K8" s="5">
+      <c r="K8" s="3">
         <v>4.77</v>
       </c>
-      <c r="L8" s="5">
+      <c r="L8" s="3">
         <v>1.91</v>
       </c>
-      <c r="M8" s="5">
+      <c r="M8" s="3">
         <v>0.119</v>
       </c>
-      <c r="N8" s="5">
+      <c r="N8" s="3">
         <v>29.02</v>
       </c>
-      <c r="O8" s="5">
+      <c r="O8" s="3">
         <v>18.7</v>
       </c>
-      <c r="P8" s="5">
+      <c r="P8" s="3">
         <v>0.483</v>
       </c>
-      <c r="Q8" s="5">
+      <c r="Q8" s="3">
         <v>2.13</v>
       </c>
-      <c r="R8" s="5">
+      <c r="R8" s="3">
         <v>2.06</v>
       </c>
-      <c r="S8" s="5">
+      <c r="S8" s="3">
         <v>0.45</v>
       </c>
-      <c r="T8" s="5">
+      <c r="T8" s="3">
         <v>125.69</v>
       </c>
-      <c r="U8" s="5">
+      <c r="U8" s="3">
         <v>5.7</v>
       </c>
-      <c r="V8" s="5">
+      <c r="V8" s="3">
         <v>0.59</v>
       </c>
-      <c r="W8" s="5">
+      <c r="W8" s="3">
         <v>27.3</v>
       </c>
     </row>
@@ -1180,70 +1168,70 @@
       <c r="A9" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="B9" s="4">
+      <c r="B9" s="2">
         <v>298</v>
       </c>
-      <c r="C9" s="5">
+      <c r="C9" s="3">
         <v>0.679</v>
       </c>
-      <c r="D9" s="5">
+      <c r="D9" s="3">
         <v>0.91</v>
       </c>
-      <c r="E9" s="5">
+      <c r="E9" s="3">
         <v>0.72</v>
       </c>
-      <c r="F9" s="5">
+      <c r="F9" s="3">
         <v>2.69</v>
       </c>
-      <c r="G9" s="4">
+      <c r="G9" s="2">
         <v>46</v>
       </c>
-      <c r="H9" s="5">
+      <c r="H9" s="3">
         <v>3.47</v>
       </c>
-      <c r="I9" s="5">
+      <c r="I9" s="3">
         <v>9.34</v>
       </c>
-      <c r="J9" s="5">
+      <c r="J9" s="3">
         <v>128.6</v>
       </c>
-      <c r="K9" s="5">
+      <c r="K9" s="3">
         <v>1.89</v>
       </c>
-      <c r="L9" s="5">
+      <c r="L9" s="3">
         <v>4.26</v>
       </c>
-      <c r="M9" s="5">
+      <c r="M9" s="3">
         <v>0.144</v>
       </c>
-      <c r="N9" s="5">
+      <c r="N9" s="3">
         <v>24.15</v>
       </c>
-      <c r="O9" s="5">
+      <c r="O9" s="3">
         <v>17.1</v>
       </c>
-      <c r="P9" s="5">
+      <c r="P9" s="3">
         <v>0.484</v>
       </c>
-      <c r="Q9" s="5">
+      <c r="Q9" s="3">
         <v>2.13</v>
       </c>
-      <c r="R9" s="5">
+      <c r="R9" s="3">
         <v>2.06</v>
       </c>
-      <c r="S9" s="5">
+      <c r="S9" s="3">
         <v>1.13</v>
       </c>
-      <c r="T9" s="5">
+      <c r="T9" s="3">
         <v>60.32</v>
       </c>
-      <c r="U9" s="5">
+      <c r="U9" s="3">
         <v>4.11</v>
       </c>
-      <c r="V9" s="5">
+      <c r="V9" s="3">
         <v>0.45</v>
       </c>
-      <c r="W9" s="4">
+      <c r="W9" s="2">
         <v>44</v>
       </c>
     </row>
@@ -1251,70 +1239,70 @@
       <c r="A10" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="B10" s="4">
+      <c r="B10" s="2">
         <v>463</v>
       </c>
-      <c r="C10" s="5">
+      <c r="C10" s="3">
         <v>0.678</v>
       </c>
-      <c r="D10" s="5">
+      <c r="D10" s="3">
         <v>0.765</v>
       </c>
-      <c r="E10" s="5">
+      <c r="E10" s="3">
         <v>0.53</v>
       </c>
-      <c r="F10" s="5">
+      <c r="F10" s="3">
         <v>3.2</v>
       </c>
-      <c r="G10" s="5">
+      <c r="G10" s="3">
         <v>61.7</v>
       </c>
-      <c r="H10" s="5">
+      <c r="H10" s="3">
         <v>3.53</v>
       </c>
-      <c r="I10" s="5">
+      <c r="I10" s="3">
         <v>11.2</v>
       </c>
-      <c r="J10" s="5">
+      <c r="J10" s="3">
         <v>183.4</v>
       </c>
-      <c r="K10" s="5">
+      <c r="K10" s="3">
         <v>4.36</v>
       </c>
-      <c r="L10" s="5">
+      <c r="L10" s="3">
         <v>2.51</v>
       </c>
-      <c r="M10" s="5">
+      <c r="M10" s="3">
         <v>0.115</v>
       </c>
-      <c r="N10" s="5">
+      <c r="N10" s="3">
         <v>30.59</v>
       </c>
-      <c r="O10" s="5">
+      <c r="O10" s="3">
         <v>19.3</v>
       </c>
-      <c r="P10" s="5">
+      <c r="P10" s="3">
         <v>0.518</v>
       </c>
-      <c r="Q10" s="5">
+      <c r="Q10" s="3">
         <v>2.15</v>
       </c>
-      <c r="R10" s="5">
+      <c r="R10" s="3">
         <v>2.07</v>
       </c>
-      <c r="S10" s="5">
+      <c r="S10" s="3">
         <v>0.49</v>
       </c>
-      <c r="T10" s="5">
+      <c r="T10" s="3">
         <v>85.25</v>
       </c>
-      <c r="U10" s="5">
+      <c r="U10" s="3">
         <v>6.39</v>
       </c>
-      <c r="V10" s="5">
+      <c r="V10" s="3">
         <v>0.54</v>
       </c>
-      <c r="W10" s="5">
+      <c r="W10" s="3">
         <v>40.7</v>
       </c>
     </row>
@@ -1322,70 +1310,70 @@
       <c r="A11" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="B11" s="4">
+      <c r="B11" s="2">
         <v>463</v>
       </c>
-      <c r="C11" s="5">
+      <c r="C11" s="3">
         <v>0.694</v>
       </c>
-      <c r="D11" s="5">
+      <c r="D11" s="3">
         <v>0.766</v>
       </c>
-      <c r="E11" s="5">
+      <c r="E11" s="3">
         <v>0.54</v>
       </c>
-      <c r="F11" s="5">
+      <c r="F11" s="3">
         <v>3.12</v>
       </c>
-      <c r="G11" s="5">
+      <c r="G11" s="3">
         <v>61.7</v>
       </c>
-      <c r="H11" s="5">
+      <c r="H11" s="3">
         <v>3.64</v>
       </c>
-      <c r="I11" s="5">
+      <c r="I11" s="3">
         <v>11.4</v>
       </c>
-      <c r="J11" s="5">
+      <c r="J11" s="3">
         <v>187.8</v>
       </c>
-      <c r="K11" s="5">
+      <c r="K11" s="3">
         <v>4.46</v>
       </c>
-      <c r="L11" s="5">
+      <c r="L11" s="3">
         <v>2.46</v>
       </c>
-      <c r="M11" s="5">
+      <c r="M11" s="3">
         <v>0.125</v>
       </c>
-      <c r="N11" s="5">
+      <c r="N11" s="3">
         <v>29.22</v>
       </c>
-      <c r="O11" s="5">
+      <c r="O11" s="3">
         <v>19.8</v>
       </c>
-      <c r="P11" s="5">
+      <c r="P11" s="3">
         <v>0.575</v>
       </c>
-      <c r="Q11" s="5">
+      <c r="Q11" s="3">
         <v>2.18</v>
       </c>
-      <c r="R11" s="5">
+      <c r="R11" s="3">
         <v>2.11</v>
       </c>
-      <c r="S11" s="5">
+      <c r="S11" s="3">
         <v>0.49</v>
       </c>
-      <c r="T11" s="5">
+      <c r="T11" s="3">
         <v>85.96</v>
       </c>
-      <c r="U11" s="5">
+      <c r="U11" s="3">
         <v>6.39</v>
       </c>
-      <c r="V11" s="5">
+      <c r="V11" s="3">
         <v>0.54</v>
       </c>
-      <c r="W11" s="5">
+      <c r="W11" s="3">
         <v>40.4</v>
       </c>
     </row>
@@ -1393,70 +1381,70 @@
       <c r="A12" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="B12" s="4">
+      <c r="B12" s="2">
         <v>413</v>
       </c>
-      <c r="C12" s="5">
+      <c r="C12" s="3">
         <v>0.678</v>
       </c>
-      <c r="D12" s="5">
+      <c r="D12" s="3">
         <v>0.791</v>
       </c>
-      <c r="E12" s="5">
+      <c r="E12" s="3">
         <v>0.59</v>
       </c>
-      <c r="F12" s="5">
+      <c r="F12" s="3">
         <v>3.1</v>
       </c>
-      <c r="G12" s="4">
+      <c r="G12" s="2">
         <v>56</v>
       </c>
-      <c r="H12" s="5">
+      <c r="H12" s="3">
         <v>3.65</v>
       </c>
-      <c r="I12" s="5">
+      <c r="I12" s="3">
         <v>11.2</v>
       </c>
-      <c r="J12" s="5">
+      <c r="J12" s="3">
         <v>183.4</v>
       </c>
-      <c r="K12" s="5">
+      <c r="K12" s="3">
         <v>4.36</v>
       </c>
-      <c r="L12" s="5">
+      <c r="L12" s="3">
         <v>2.6</v>
       </c>
-      <c r="M12" s="5">
+      <c r="M12" s="3">
         <v>0.145</v>
       </c>
-      <c r="N12" s="5">
+      <c r="N12" s="3">
         <v>25.21</v>
       </c>
-      <c r="O12" s="5">
+      <c r="O12" s="3">
         <v>18.1</v>
       </c>
-      <c r="P12" s="5">
+      <c r="P12" s="3">
         <v>0.58</v>
       </c>
-      <c r="Q12" s="5">
+      <c r="Q12" s="3">
         <v>2.19</v>
       </c>
-      <c r="R12" s="5">
+      <c r="R12" s="3">
         <v>2.11</v>
       </c>
-      <c r="S12" s="5">
+      <c r="S12" s="3">
         <v>0.5</v>
       </c>
-      <c r="T12" s="5">
+      <c r="T12" s="3">
         <v>83.84</v>
       </c>
-      <c r="U12" s="5">
+      <c r="U12" s="3">
         <v>5.7</v>
       </c>
-      <c r="V12" s="5">
+      <c r="V12" s="3">
         <v>0.53</v>
       </c>
-      <c r="W12" s="5">
+      <c r="W12" s="3">
         <v>38.2</v>
       </c>
     </row>
@@ -1464,70 +1452,70 @@
       <c r="A13" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="B13" s="4">
+      <c r="B13" s="2">
         <v>348</v>
       </c>
-      <c r="C13" s="5">
+      <c r="C13" s="3">
         <v>0.678</v>
       </c>
-      <c r="D13" s="5">
+      <c r="D13" s="3">
         <v>0.825</v>
       </c>
-      <c r="E13" s="5">
+      <c r="E13" s="3">
         <v>0.6</v>
       </c>
-      <c r="F13" s="5">
+      <c r="F13" s="3">
         <v>2.97</v>
       </c>
-      <c r="G13" s="5">
+      <c r="G13" s="3">
         <v>51.9</v>
       </c>
-      <c r="H13" s="5">
+      <c r="H13" s="3">
         <v>3.81</v>
       </c>
-      <c r="I13" s="5">
+      <c r="I13" s="3">
         <v>11.2</v>
       </c>
-      <c r="J13" s="5">
+      <c r="J13" s="3">
         <v>183.4</v>
       </c>
-      <c r="K13" s="5">
+      <c r="K13" s="3">
         <v>4.36</v>
       </c>
-      <c r="L13" s="5">
+      <c r="L13" s="3">
         <v>2.71</v>
       </c>
-      <c r="M13" s="5">
+      <c r="M13" s="3">
         <v>0.175</v>
       </c>
-      <c r="N13" s="5">
+      <c r="N13" s="3">
         <v>21.7</v>
       </c>
-      <c r="O13" s="5">
+      <c r="O13" s="3">
         <v>17.5</v>
       </c>
-      <c r="P13" s="5">
+      <c r="P13" s="3">
         <v>0.656</v>
       </c>
-      <c r="Q13" s="5">
+      <c r="Q13" s="3">
         <v>2.23</v>
       </c>
-      <c r="R13" s="5">
+      <c r="R13" s="3">
         <v>2.16</v>
       </c>
-      <c r="S13" s="5">
+      <c r="S13" s="3">
         <v>0.51</v>
       </c>
-      <c r="T13" s="5">
+      <c r="T13" s="3">
         <v>82.08</v>
       </c>
-      <c r="U13" s="5">
+      <c r="U13" s="3">
         <v>4.8</v>
       </c>
-      <c r="V13" s="5">
+      <c r="V13" s="3">
         <v>0.52</v>
       </c>
-      <c r="W13" s="5">
+      <c r="W13" s="3">
         <v>34.3</v>
       </c>
     </row>
@@ -1535,70 +1523,70 @@
       <c r="A14" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="B14" s="4">
+      <c r="B14" s="2">
         <v>298</v>
       </c>
-      <c r="C14" s="5">
+      <c r="C14" s="3">
         <v>0.678</v>
       </c>
-      <c r="D14" s="5">
+      <c r="D14" s="3">
         <v>0.852</v>
       </c>
-      <c r="E14" s="5">
+      <c r="E14" s="3">
         <v>0.6</v>
       </c>
-      <c r="F14" s="5">
+      <c r="F14" s="3">
         <v>2.87</v>
       </c>
-      <c r="G14" s="5">
+      <c r="G14" s="3">
         <v>48.8</v>
       </c>
-      <c r="H14" s="5">
+      <c r="H14" s="3">
         <v>3.92</v>
       </c>
-      <c r="I14" s="5">
+      <c r="I14" s="3">
         <v>11.2</v>
       </c>
-      <c r="J14" s="5">
+      <c r="J14" s="3">
         <v>183.4</v>
       </c>
-      <c r="K14" s="5">
+      <c r="K14" s="3">
         <v>4.36</v>
       </c>
-      <c r="L14" s="5">
+      <c r="L14" s="3">
         <v>2.79</v>
       </c>
-      <c r="M14" s="5">
+      <c r="M14" s="3">
         <v>0.205</v>
       </c>
-      <c r="N14" s="5">
+      <c r="N14" s="3">
         <v>19.15</v>
       </c>
-      <c r="O14" s="4">
+      <c r="O14" s="2">
         <v>17</v>
       </c>
-      <c r="P14" s="5">
+      <c r="P14" s="3">
         <v>0.708</v>
       </c>
-      <c r="Q14" s="5">
+      <c r="Q14" s="3">
         <v>2.27</v>
       </c>
-      <c r="R14" s="5">
+      <c r="R14" s="3">
         <v>2.19</v>
       </c>
-      <c r="S14" s="5">
+      <c r="S14" s="3">
         <v>0.52</v>
       </c>
-      <c r="T14" s="5">
+      <c r="T14" s="3">
         <v>80.84</v>
       </c>
-      <c r="U14" s="5">
+      <c r="U14" s="3">
         <v>4.11</v>
       </c>
-      <c r="V14" s="5">
+      <c r="V14" s="3">
         <v>0.51</v>
       </c>
-      <c r="W14" s="5">
+      <c r="W14" s="3">
         <v>30.7</v>
       </c>
     </row>
@@ -1606,70 +1594,70 @@
       <c r="A15" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="B15" s="4">
+      <c r="B15" s="2">
         <v>298</v>
       </c>
-      <c r="C15" s="5">
+      <c r="C15" s="3">
         <v>0.57</v>
       </c>
-      <c r="D15" s="5">
+      <c r="D15" s="3">
         <v>0.918</v>
       </c>
-      <c r="E15" s="5">
+      <c r="E15" s="3">
         <v>0.43</v>
       </c>
-      <c r="F15" s="5">
+      <c r="F15" s="3">
         <v>3.17</v>
       </c>
-      <c r="G15" s="5">
+      <c r="G15" s="3">
         <v>55.2</v>
       </c>
-      <c r="H15" s="5">
+      <c r="H15" s="3">
         <v>3.94</v>
       </c>
-      <c r="I15" s="5">
+      <c r="I15" s="3">
         <v>12.5</v>
       </c>
-      <c r="J15" s="5">
+      <c r="J15" s="3">
         <v>274.2</v>
       </c>
-      <c r="K15" s="5">
+      <c r="K15" s="3">
         <v>4.89</v>
       </c>
-      <c r="L15" s="5">
+      <c r="L15" s="3">
         <v>2.02</v>
       </c>
-      <c r="M15" s="5">
+      <c r="M15" s="3">
         <v>0.202</v>
       </c>
-      <c r="N15" s="5">
+      <c r="N15" s="3">
         <v>19.52</v>
       </c>
-      <c r="O15" s="5">
+      <c r="O15" s="3">
         <v>17.4</v>
       </c>
-      <c r="P15" s="5">
+      <c r="P15" s="3">
         <v>0.714</v>
       </c>
-      <c r="Q15" s="5">
+      <c r="Q15" s="3">
         <v>2.27</v>
       </c>
-      <c r="R15" s="5">
+      <c r="R15" s="3">
         <v>2.19</v>
       </c>
-      <c r="S15" s="5">
+      <c r="S15" s="3">
         <v>0.47</v>
       </c>
-      <c r="T15" s="5">
+      <c r="T15" s="3">
         <v>120.66</v>
       </c>
-      <c r="U15" s="5">
+      <c r="U15" s="3">
         <v>4.11</v>
       </c>
-      <c r="V15" s="5">
+      <c r="V15" s="3">
         <v>0.57</v>
       </c>
-      <c r="W15" s="5">
+      <c r="W15" s="3">
         <v>22.2</v>
       </c>
     </row>
@@ -1677,70 +1665,70 @@
       <c r="A16" s="1" t="s">
         <v>37</v>
       </c>
-      <c r="B16" s="4">
+      <c r="B16" s="2">
         <v>413</v>
       </c>
-      <c r="C16" s="5">
+      <c r="C16" s="3">
         <v>0.39</v>
       </c>
-      <c r="D16" s="5">
+      <c r="D16" s="3">
         <v>1.13</v>
       </c>
-      <c r="E16" s="5">
+      <c r="E16" s="3">
         <v>0.39</v>
       </c>
-      <c r="F16" s="4">
+      <c r="F16" s="2">
         <v>377</v>
       </c>
-      <c r="G16" s="5">
+      <c r="G16" s="3">
         <v>62.5</v>
       </c>
-      <c r="H16" s="5">
+      <c r="H16" s="3">
         <v>4.07</v>
       </c>
-      <c r="I16" s="5">
+      <c r="I16" s="3">
         <v>15.3</v>
       </c>
-      <c r="J16" s="4">
+      <c r="J16" s="2">
         <v>598</v>
       </c>
-      <c r="K16" s="5">
+      <c r="K16" s="3">
         <v>5.97</v>
       </c>
-      <c r="L16" s="5">
+      <c r="L16" s="3">
         <v>1.14</v>
       </c>
-      <c r="M16" s="5">
+      <c r="M16" s="3">
         <v>0.243</v>
       </c>
-      <c r="N16" s="5">
+      <c r="N16" s="3">
         <v>16.72</v>
       </c>
-      <c r="O16" s="5">
+      <c r="O16" s="3">
         <v>16.6</v>
       </c>
-      <c r="P16" s="5">
+      <c r="P16" s="3">
         <v>0.77</v>
       </c>
-      <c r="Q16" s="5">
+      <c r="Q16" s="3">
         <v>2.31</v>
       </c>
-      <c r="R16" s="5">
+      <c r="R16" s="3">
         <v>2.23</v>
       </c>
-      <c r="S16" s="5">
+      <c r="S16" s="3">
         <v>0.39</v>
       </c>
-      <c r="T16" s="5">
+      <c r="T16" s="3">
         <v>258.82</v>
       </c>
-      <c r="U16" s="5">
+      <c r="U16" s="3">
         <v>5.7</v>
       </c>
-      <c r="V16" s="5">
+      <c r="V16" s="3">
         <v>0.69</v>
       </c>
-      <c r="W16" s="5">
+      <c r="W16" s="3">
         <v>17.6</v>
       </c>
     </row>
@@ -1748,70 +1736,70 @@
       <c r="A17" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="B17" s="4">
+      <c r="B17" s="2">
         <v>413</v>
       </c>
-      <c r="C17" s="5">
+      <c r="C17" s="3">
         <v>0.42</v>
       </c>
-      <c r="D17" s="5">
+      <c r="D17" s="3">
         <v>0.969</v>
       </c>
-      <c r="E17" s="5">
+      <c r="E17" s="3">
         <v>0.24</v>
       </c>
-      <c r="F17" s="5">
+      <c r="F17" s="3">
         <v>4.08</v>
       </c>
-      <c r="G17" s="5">
+      <c r="G17" s="3">
         <v>76.7</v>
       </c>
-      <c r="H17" s="5">
+      <c r="H17" s="3">
         <v>4.19</v>
       </c>
-      <c r="I17" s="5">
+      <c r="I17" s="3">
         <v>17.11</v>
       </c>
-      <c r="J17" s="5">
+      <c r="J17" s="3">
         <v>697.12</v>
       </c>
-      <c r="K17" s="5">
+      <c r="K17" s="3">
         <v>6.69</v>
       </c>
-      <c r="L17" s="5">
+      <c r="L17" s="3">
         <v>0.84</v>
       </c>
-      <c r="M17" s="5">
+      <c r="M17" s="3">
         <v>0.209</v>
       </c>
-      <c r="N17" s="5">
+      <c r="N17" s="3">
         <v>20.1</v>
       </c>
-      <c r="O17" s="5">
+      <c r="O17" s="3">
         <v>18.8</v>
       </c>
-      <c r="P17" s="5">
+      <c r="P17" s="3">
         <v>0.819</v>
       </c>
-      <c r="Q17" s="5">
+      <c r="Q17" s="3">
         <v>2.35</v>
       </c>
-      <c r="R17" s="5">
+      <c r="R17" s="3">
         <v>2.26</v>
       </c>
-      <c r="S17" s="5">
+      <c r="S17" s="3">
         <v>0.35</v>
       </c>
-      <c r="T17" s="5">
+      <c r="T17" s="3">
         <v>297.22</v>
       </c>
-      <c r="U17" s="5">
+      <c r="U17" s="3">
         <v>5.7</v>
       </c>
-      <c r="V17" s="5">
+      <c r="V17" s="3">
         <v>0.76</v>
       </c>
-      <c r="W17" s="5">
+      <c r="W17" s="3">
         <v>13.2</v>
       </c>
     </row>
@@ -1819,70 +1807,70 @@
       <c r="A18" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="B18" s="4">
+      <c r="B18" s="2">
         <v>298</v>
       </c>
-      <c r="C18" s="5">
+      <c r="C18" s="3">
         <v>0.436</v>
       </c>
-      <c r="D18" s="5">
+      <c r="D18" s="3">
         <v>1.11</v>
       </c>
-      <c r="E18" s="5">
+      <c r="E18" s="3">
         <v>0.31</v>
       </c>
-      <c r="F18" s="5">
+      <c r="F18" s="3">
         <v>3.43</v>
       </c>
-      <c r="G18" s="5">
+      <c r="G18" s="3">
         <v>61.9</v>
       </c>
-      <c r="H18" s="5">
+      <c r="H18" s="3">
         <v>4.29</v>
       </c>
-      <c r="I18" s="5">
+      <c r="I18" s="3">
         <v>14.7</v>
       </c>
-      <c r="J18" s="5">
+      <c r="J18" s="3">
         <v>494.6</v>
       </c>
-      <c r="K18" s="5">
+      <c r="K18" s="3">
         <v>5.75</v>
       </c>
-      <c r="L18" s="5">
+      <c r="L18" s="3">
         <v>1.35</v>
       </c>
-      <c r="M18" s="5">
+      <c r="M18" s="3">
         <v>0.241</v>
       </c>
-      <c r="N18" s="5">
+      <c r="N18" s="3">
         <v>17.79</v>
       </c>
-      <c r="O18" s="5">
+      <c r="O18" s="3">
         <v>18.1</v>
       </c>
-      <c r="P18" s="5">
+      <c r="P18" s="3">
         <v>0.856</v>
       </c>
-      <c r="Q18" s="5">
+      <c r="Q18" s="3">
         <v>2.37</v>
       </c>
-      <c r="R18" s="5">
+      <c r="R18" s="3">
         <v>2.29</v>
       </c>
-      <c r="S18" s="5">
+      <c r="S18" s="3">
         <v>0.41</v>
       </c>
-      <c r="T18" s="5">
+      <c r="T18" s="3">
         <v>208.42</v>
       </c>
-      <c r="U18" s="5">
+      <c r="U18" s="3">
         <v>4.11</v>
       </c>
-      <c r="V18" s="5">
+      <c r="V18" s="3">
         <v>0.64</v>
       </c>
-      <c r="W18" s="5">
+      <c r="W18" s="3">
         <v>15.6</v>
       </c>
     </row>
@@ -1890,70 +1878,70 @@
       <c r="A19" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="B19" s="4">
+      <c r="B19" s="2">
         <v>298</v>
       </c>
-      <c r="C19" s="5">
+      <c r="C19" s="3">
         <v>0.563</v>
       </c>
-      <c r="D19" s="5">
+      <c r="D19" s="3">
         <v>0.89</v>
       </c>
-      <c r="E19" s="5">
+      <c r="E19" s="3">
         <v>0.46</v>
       </c>
-      <c r="F19" s="5">
+      <c r="F19" s="3">
         <v>3.31</v>
       </c>
-      <c r="G19" s="5">
+      <c r="G19" s="3">
         <v>51.8</v>
       </c>
-      <c r="H19" s="5">
+      <c r="H19" s="3">
         <v>4.53</v>
       </c>
-      <c r="I19" s="4">
+      <c r="I19" s="2">
         <v>15</v>
       </c>
-      <c r="J19" s="5">
+      <c r="J19" s="3">
         <v>399.3</v>
       </c>
-      <c r="K19" s="5">
+      <c r="K19" s="3">
         <v>5.86</v>
       </c>
-      <c r="L19" s="5">
+      <c r="L19" s="3">
         <v>1.34</v>
       </c>
-      <c r="M19" s="5">
+      <c r="M19" s="3">
         <v>0.379</v>
       </c>
-      <c r="N19" s="5">
+      <c r="N19" s="3">
         <v>11.94</v>
       </c>
-      <c r="O19" s="5">
+      <c r="O19" s="3">
         <v>15.6</v>
       </c>
-      <c r="P19" s="5">
+      <c r="P19" s="3">
         <v>0.941</v>
       </c>
-      <c r="Q19" s="5">
+      <c r="Q19" s="3">
         <v>2.44</v>
       </c>
-      <c r="R19" s="5">
+      <c r="R19" s="3">
         <v>2.35</v>
       </c>
-      <c r="S19" s="5">
+      <c r="S19" s="3">
         <v>0.42</v>
       </c>
-      <c r="T19" s="5">
+      <c r="T19" s="3">
         <v>163.78</v>
       </c>
-      <c r="U19" s="5">
+      <c r="U19" s="3">
         <v>4.11</v>
       </c>
-      <c r="V19" s="5">
+      <c r="V19" s="3">
         <v>0.64</v>
       </c>
-      <c r="W19" s="5">
+      <c r="W19" s="3">
         <v>15.9</v>
       </c>
     </row>
@@ -1961,70 +1949,70 @@
       <c r="A20" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="B20" s="4">
+      <c r="B20" s="2">
         <v>298</v>
       </c>
-      <c r="C20" s="5">
+      <c r="C20" s="3">
         <v>0.841</v>
       </c>
-      <c r="D20" s="5">
+      <c r="D20" s="3">
         <v>0.895</v>
       </c>
-      <c r="E20" s="5">
+      <c r="E20" s="3">
         <v>1.34</v>
       </c>
-      <c r="F20" s="5">
+      <c r="F20" s="3">
         <v>2.21</v>
       </c>
-      <c r="G20" s="5">
+      <c r="G20" s="3">
         <v>37.3</v>
       </c>
-      <c r="H20" s="5">
+      <c r="H20" s="3">
         <v>4.54</v>
       </c>
-      <c r="I20" s="5">
+      <c r="I20" s="3">
         <v>10.1</v>
       </c>
-      <c r="J20" s="5">
+      <c r="J20" s="3">
         <v>122.4</v>
       </c>
-      <c r="K20" s="5">
+      <c r="K20" s="3">
         <v>2.26</v>
       </c>
-      <c r="L20" s="5">
+      <c r="L20" s="3">
         <v>4.41</v>
       </c>
-      <c r="M20" s="5">
+      <c r="M20" s="3">
         <v>0.335</v>
       </c>
-      <c r="N20" s="5">
+      <c r="N20" s="3">
         <v>13.55</v>
       </c>
-      <c r="O20" s="5">
+      <c r="O20" s="3">
         <v>16.9</v>
       </c>
-      <c r="P20" s="5">
+      <c r="P20" s="3">
         <v>0.944</v>
       </c>
-      <c r="Q20" s="5">
+      <c r="Q20" s="3">
         <v>2.44</v>
       </c>
-      <c r="R20" s="5">
+      <c r="R20" s="3">
         <v>2.35</v>
       </c>
-      <c r="S20" s="5">
+      <c r="S20" s="3">
         <v>1.08</v>
       </c>
-      <c r="T20" s="5">
+      <c r="T20" s="3">
         <v>50.16</v>
       </c>
-      <c r="U20" s="5">
+      <c r="U20" s="3">
         <v>4.11</v>
       </c>
-      <c r="V20" s="5">
+      <c r="V20" s="3">
         <v>0.43</v>
       </c>
-      <c r="W20" s="5">
+      <c r="W20" s="3">
         <v>52.2</v>
       </c>
     </row>
@@ -2032,70 +2020,70 @@
       <c r="A21" s="1" t="s">
         <v>42</v>
       </c>
-      <c r="B21" s="4">
+      <c r="B21" s="2">
         <v>413</v>
       </c>
-      <c r="C21" s="5">
+      <c r="C21" s="3">
         <v>0.437</v>
       </c>
-      <c r="D21" s="5">
+      <c r="D21" s="3">
         <v>0.969</v>
       </c>
-      <c r="E21" s="5">
+      <c r="E21" s="3">
         <v>0.25</v>
       </c>
-      <c r="F21" s="5">
+      <c r="F21" s="3">
         <v>3.92</v>
       </c>
-      <c r="G21" s="5">
+      <c r="G21" s="3">
         <v>76.3</v>
       </c>
-      <c r="H21" s="5">
+      <c r="H21" s="3">
         <v>4.54</v>
       </c>
-      <c r="I21" s="5">
+      <c r="I21" s="3">
         <v>17.8</v>
       </c>
-      <c r="J21" s="5">
+      <c r="J21" s="3">
         <v>725.34</v>
       </c>
-      <c r="K21" s="5">
+      <c r="K21" s="3">
         <v>6.96</v>
       </c>
-      <c r="L21" s="5">
+      <c r="L21" s="3">
         <v>0.8</v>
       </c>
-      <c r="M21" s="5">
+      <c r="M21" s="3">
         <v>0.247</v>
       </c>
-      <c r="N21" s="5">
+      <c r="N21" s="3">
         <v>18.35</v>
       </c>
-      <c r="O21" s="5">
+      <c r="O21" s="3">
         <v>19.4</v>
       </c>
-      <c r="P21" s="5">
+      <c r="P21" s="3">
         <v>0.944</v>
       </c>
-      <c r="Q21" s="5">
+      <c r="Q21" s="3">
         <v>2.44</v>
       </c>
-      <c r="R21" s="5">
+      <c r="R21" s="3">
         <v>2.35</v>
       </c>
-      <c r="S21" s="5">
+      <c r="S21" s="3">
         <v>0.35</v>
       </c>
-      <c r="T21" s="5">
+      <c r="T21" s="3">
         <v>297.19</v>
       </c>
-      <c r="U21" s="5">
+      <c r="U21" s="3">
         <v>5.7</v>
       </c>
-      <c r="V21" s="5">
+      <c r="V21" s="3">
         <v>0.76</v>
       </c>
-      <c r="W21" s="5">
+      <c r="W21" s="3">
         <v>13.2</v>
       </c>
     </row>
@@ -2103,70 +2091,70 @@
       <c r="A22" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="B22" s="4">
+      <c r="B22" s="2">
         <v>300</v>
       </c>
-      <c r="C22" s="5">
+      <c r="C22" s="3">
         <v>0.661</v>
       </c>
-      <c r="D22" s="5">
+      <c r="D22" s="3">
         <v>0.89</v>
       </c>
-      <c r="E22" s="5">
+      <c r="E22" s="3">
         <v>0.71</v>
       </c>
-      <c r="F22" s="5">
+      <c r="F22" s="3">
         <v>2.82</v>
       </c>
-      <c r="G22" s="5">
+      <c r="G22" s="3">
         <v>45.4</v>
       </c>
-      <c r="H22" s="5">
+      <c r="H22" s="3">
         <v>4.83</v>
       </c>
-      <c r="I22" s="5">
+      <c r="I22" s="3">
         <v>13.7</v>
       </c>
-      <c r="J22" s="5">
+      <c r="J22" s="3">
         <v>284.8</v>
       </c>
-      <c r="K22" s="5">
+      <c r="K22" s="3">
         <v>5.27</v>
       </c>
-      <c r="L22" s="5">
+      <c r="L22" s="3">
         <v>1.88</v>
       </c>
-      <c r="M22" s="5">
+      <c r="M22" s="3">
         <v>0.442</v>
       </c>
-      <c r="N22" s="5">
+      <c r="N22" s="3">
         <v>10.93</v>
       </c>
-      <c r="O22" s="5">
+      <c r="O22" s="3">
         <v>16.1</v>
       </c>
-      <c r="P22" s="5">
+      <c r="P22" s="3">
         <v>1.039</v>
       </c>
-      <c r="Q22" s="5">
+      <c r="Q22" s="3">
         <v>2.52</v>
       </c>
-      <c r="R22" s="5">
+      <c r="R22" s="3">
         <v>2.43</v>
       </c>
-      <c r="S22" s="5">
+      <c r="S22" s="3">
         <v>0.48</v>
       </c>
-      <c r="T22" s="5">
+      <c r="T22" s="3">
         <v>113.08</v>
       </c>
-      <c r="U22" s="5">
+      <c r="U22" s="3">
         <v>4.14</v>
       </c>
-      <c r="V22" s="5">
+      <c r="V22" s="3">
         <v>0.56</v>
       </c>
-      <c r="W22" s="5">
+      <c r="W22" s="3">
         <v>23.1</v>
       </c>
     </row>
@@ -2174,70 +2162,70 @@
       <c r="A23" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="B23" s="4">
+      <c r="B23" s="2">
         <v>353</v>
       </c>
-      <c r="C23" s="5">
+      <c r="C23" s="3">
         <v>0.805</v>
       </c>
-      <c r="D23" s="5">
+      <c r="D23" s="3">
         <v>1.06</v>
       </c>
-      <c r="E23" s="5">
+      <c r="E23" s="3">
         <v>2.25</v>
       </c>
-      <c r="F23" s="5">
+      <c r="F23" s="3">
         <v>1.95</v>
       </c>
-      <c r="G23" s="5">
+      <c r="G23" s="3">
         <v>33.4</v>
       </c>
-      <c r="H23" s="5">
+      <c r="H23" s="3">
         <v>4.99</v>
       </c>
-      <c r="I23" s="5">
+      <c r="I23" s="3">
         <v>9.71</v>
       </c>
-      <c r="J23" s="5">
+      <c r="J23" s="3">
         <v>117.12</v>
       </c>
-      <c r="K23" s="5">
+      <c r="K23" s="3">
         <v>2.66</v>
       </c>
       <c r="L23" s="3" t="s">
         <v>45</v>
       </c>
-      <c r="M23" s="5">
+      <c r="M23" s="3">
         <v>0.423</v>
       </c>
-      <c r="N23" s="5">
+      <c r="N23" s="3">
         <v>11.81</v>
       </c>
-      <c r="O23" s="5">
+      <c r="O23" s="3">
         <v>17.1</v>
       </c>
-      <c r="P23" s="5">
+      <c r="P23" s="3">
         <v>1.086</v>
       </c>
-      <c r="Q23" s="5">
+      <c r="Q23" s="3">
         <v>2.56</v>
       </c>
-      <c r="R23" s="5">
+      <c r="R23" s="3">
         <v>2.47</v>
       </c>
-      <c r="S23" s="5">
+      <c r="S23" s="3">
         <v>0.96</v>
       </c>
-      <c r="T23" s="5">
+      <c r="T23" s="3">
         <v>45.77</v>
       </c>
-      <c r="U23" s="5">
+      <c r="U23" s="3">
         <v>4.87</v>
       </c>
-      <c r="V23" s="5">
+      <c r="V23" s="3">
         <v>0.39</v>
       </c>
-      <c r="W23" s="5">
+      <c r="W23" s="3">
         <v>80.2</v>
       </c>
     </row>
@@ -2245,70 +2233,70 @@
       <c r="A24" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="B24" s="4">
+      <c r="B24" s="2">
         <v>473</v>
       </c>
-      <c r="C24" s="5">
+      <c r="C24" s="3">
         <v>0.763</v>
       </c>
-      <c r="D24" s="5">
+      <c r="D24" s="3">
         <v>1.14</v>
       </c>
-      <c r="E24" s="5">
+      <c r="E24" s="3">
         <v>2.12</v>
       </c>
-      <c r="F24" s="5">
+      <c r="F24" s="3">
         <v>1.91</v>
       </c>
-      <c r="G24" s="5">
+      <c r="G24" s="3">
         <v>40.1</v>
       </c>
-      <c r="H24" s="5">
+      <c r="H24" s="3">
         <v>5.06</v>
       </c>
-      <c r="I24" s="5">
+      <c r="I24" s="3">
         <v>9.65</v>
       </c>
-      <c r="J24" s="5">
+      <c r="J24" s="3">
         <v>122.11</v>
       </c>
-      <c r="K24" s="5">
+      <c r="K24" s="3">
         <v>4.07</v>
       </c>
-      <c r="L24" s="5">
+      <c r="L24" s="3">
         <v>5.62</v>
       </c>
-      <c r="M24" s="5">
+      <c r="M24" s="3">
         <v>0.293</v>
       </c>
-      <c r="N24" s="5">
+      <c r="N24" s="3">
         <v>17.28</v>
       </c>
-      <c r="O24" s="4">
+      <c r="O24" s="2">
         <v>21</v>
       </c>
-      <c r="P24" s="5">
+      <c r="P24" s="3">
         <v>1.105</v>
       </c>
-      <c r="Q24" s="5">
+      <c r="Q24" s="3">
         <v>2.58</v>
       </c>
-      <c r="R24" s="5">
+      <c r="R24" s="3">
         <v>2.48</v>
       </c>
-      <c r="S24" s="5">
+      <c r="S24" s="3">
         <v>0.63</v>
       </c>
-      <c r="T24" s="5">
+      <c r="T24" s="3">
         <v>47.4</v>
       </c>
-      <c r="U24" s="5">
+      <c r="U24" s="3">
         <v>6.53</v>
       </c>
-      <c r="V24" s="5">
+      <c r="V24" s="3">
         <v>0.39</v>
       </c>
-      <c r="W24" s="5">
+      <c r="W24" s="3">
         <v>111.5</v>
       </c>
     </row>
@@ -2316,70 +2304,70 @@
       <c r="A25" s="1" t="s">
         <v>47</v>
       </c>
-      <c r="B25" s="4">
+      <c r="B25" s="2">
         <v>373</v>
       </c>
-      <c r="C25" s="5">
+      <c r="C25" s="3">
         <v>0.366</v>
       </c>
-      <c r="D25" s="5">
+      <c r="D25" s="3">
         <v>0.96</v>
       </c>
-      <c r="E25" s="5">
+      <c r="E25" s="3">
         <v>0.11</v>
       </c>
-      <c r="F25" s="5">
+      <c r="F25" s="3">
         <v>4.73</v>
       </c>
-      <c r="G25" s="5">
+      <c r="G25" s="3">
         <v>98.4</v>
       </c>
-      <c r="H25" s="5">
+      <c r="H25" s="3">
         <v>5.19</v>
       </c>
-      <c r="I25" s="5">
+      <c r="I25" s="3">
         <v>24.4</v>
       </c>
-      <c r="J25" s="4">
+      <c r="J25" s="2">
         <v>1622</v>
       </c>
-      <c r="K25" s="5">
+      <c r="K25" s="3">
         <v>9.53</v>
       </c>
-      <c r="L25" s="5">
+      <c r="L25" s="3">
         <v>0.36</v>
       </c>
-      <c r="M25" s="5">
+      <c r="M25" s="3">
         <v>0.317</v>
       </c>
-      <c r="N25" s="5">
+      <c r="N25" s="3">
         <v>16.35</v>
       </c>
-      <c r="O25" s="5">
+      <c r="O25" s="3">
         <v>20.8</v>
       </c>
-      <c r="P25" s="5">
+      <c r="P25" s="3">
         <v>1.143</v>
       </c>
-      <c r="Q25" s="5">
+      <c r="Q25" s="3">
         <v>2.61</v>
       </c>
-      <c r="R25" s="5">
+      <c r="R25" s="3">
         <v>2.52</v>
       </c>
-      <c r="S25" s="5">
+      <c r="S25" s="3">
         <v>0.27</v>
       </c>
-      <c r="T25" s="5">
+      <c r="T25" s="3">
         <v>621.59</v>
       </c>
-      <c r="U25" s="5">
+      <c r="U25" s="3">
         <v>5.15</v>
       </c>
-      <c r="V25" s="5">
+      <c r="V25" s="3">
         <v>0.97</v>
       </c>
-      <c r="W25" s="5">
+      <c r="W25" s="3">
         <v>5.7</v>
       </c>
     </row>
@@ -2387,70 +2375,70 @@
       <c r="A26" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="B26" s="4">
+      <c r="B26" s="2">
         <v>333</v>
       </c>
-      <c r="C26" s="5">
+      <c r="C26" s="3">
         <v>0.49</v>
       </c>
-      <c r="D26" s="5">
+      <c r="D26" s="3">
         <v>1.08</v>
       </c>
-      <c r="E26" s="5">
+      <c r="E26" s="3">
         <v>0.44</v>
       </c>
-      <c r="F26" s="5">
+      <c r="F26" s="3">
         <v>3.14</v>
       </c>
-      <c r="G26" s="5">
+      <c r="G26" s="3">
         <v>57.9</v>
       </c>
-      <c r="H26" s="5">
+      <c r="H26" s="3">
         <v>5.26</v>
       </c>
-      <c r="I26" s="5">
+      <c r="I26" s="3">
         <v>16.5</v>
       </c>
       <c r="J26" s="3" t="s">
         <v>49</v>
       </c>
-      <c r="K26" s="5">
+      <c r="K26" s="3">
         <v>6.45</v>
       </c>
-      <c r="L26" s="5">
+      <c r="L26" s="3">
         <v>1.17</v>
       </c>
-      <c r="M26" s="5">
+      <c r="M26" s="3">
         <v>0.428</v>
       </c>
-      <c r="N26" s="5">
+      <c r="N26" s="3">
         <v>12.3</v>
       </c>
-      <c r="O26" s="5">
+      <c r="O26" s="3">
         <v>18.4</v>
       </c>
-      <c r="P26" s="5">
+      <c r="P26" s="3">
         <v>1.162</v>
       </c>
-      <c r="Q26" s="5">
+      <c r="Q26" s="3">
         <v>2.63</v>
       </c>
-      <c r="R26" s="5">
+      <c r="R26" s="3">
         <v>2.53</v>
       </c>
-      <c r="S26" s="5">
+      <c r="S26" s="3">
         <v>0.41</v>
       </c>
-      <c r="T26" s="5">
+      <c r="T26" s="3">
         <v>211.52</v>
       </c>
-      <c r="U26" s="5">
+      <c r="U26" s="3">
         <v>4.6</v>
       </c>
-      <c r="V26" s="5">
+      <c r="V26" s="3">
         <v>0.65</v>
       </c>
-      <c r="W26" s="5">
+      <c r="W26" s="3">
         <v>16.7</v>
       </c>
     </row>
@@ -2458,70 +2446,70 @@
       <c r="A27" s="1" t="s">
         <v>50</v>
       </c>
-      <c r="B27" s="4">
+      <c r="B27" s="2">
         <v>298</v>
       </c>
-      <c r="C27" s="5">
+      <c r="C27" s="3">
         <v>0.818</v>
       </c>
-      <c r="D27" s="5">
+      <c r="D27" s="3">
         <v>0.913</v>
       </c>
-      <c r="E27" s="5">
+      <c r="E27" s="3">
         <v>0.98</v>
       </c>
-      <c r="F27" s="5">
+      <c r="F27" s="3">
         <v>2.22</v>
       </c>
-      <c r="G27" s="5">
+      <c r="G27" s="3">
         <v>43.6</v>
       </c>
-      <c r="H27" s="5">
+      <c r="H27" s="3">
         <v>5.33</v>
       </c>
-      <c r="I27" s="5">
+      <c r="I27" s="3">
         <v>11.9</v>
       </c>
-      <c r="J27" s="5">
+      <c r="J27" s="3">
         <v>173.6</v>
       </c>
-      <c r="K27" s="5">
+      <c r="K27" s="3">
         <v>2.61</v>
       </c>
-      <c r="L27" s="5">
+      <c r="L27" s="3">
         <v>3.16</v>
       </c>
-      <c r="M27" s="5">
+      <c r="M27" s="3">
         <v>0.399</v>
       </c>
-      <c r="N27" s="5">
+      <c r="N27" s="3">
         <v>13.35</v>
       </c>
-      <c r="O27" s="5">
+      <c r="O27" s="3">
         <v>19.6</v>
       </c>
-      <c r="P27" s="5">
+      <c r="P27" s="3">
         <v>1.182</v>
       </c>
-      <c r="Q27" s="5">
+      <c r="Q27" s="3">
         <v>2.65</v>
       </c>
-      <c r="R27" s="5">
+      <c r="R27" s="3">
         <v>2.55</v>
       </c>
-      <c r="S27" s="5">
+      <c r="S27" s="3">
         <v>1.01</v>
       </c>
-      <c r="T27" s="5">
+      <c r="T27" s="3">
         <v>65.62</v>
       </c>
-      <c r="U27" s="5">
+      <c r="U27" s="3">
         <v>4.11</v>
       </c>
-      <c r="V27" s="5">
+      <c r="V27" s="3">
         <v>0.47</v>
       </c>
-      <c r="W27" s="5">
+      <c r="W27" s="3">
         <v>40.6</v>
       </c>
     </row>
@@ -2529,70 +2517,70 @@
       <c r="A28" s="1" t="s">
         <v>51</v>
       </c>
-      <c r="B28" s="4">
+      <c r="B28" s="2">
         <v>543</v>
       </c>
-      <c r="C28" s="5">
+      <c r="C28" s="3">
         <v>0.853</v>
       </c>
-      <c r="D28" s="5">
+      <c r="D28" s="3">
         <v>0.985</v>
       </c>
-      <c r="E28" s="5">
+      <c r="E28" s="3">
         <v>2.25</v>
       </c>
-      <c r="F28" s="5">
+      <c r="F28" s="3">
         <v>1.98</v>
       </c>
-      <c r="G28" s="5">
+      <c r="G28" s="3">
         <v>41.1</v>
       </c>
-      <c r="H28" s="5">
+      <c r="H28" s="3">
         <v>5.53</v>
       </c>
-      <c r="I28" s="5">
+      <c r="I28" s="3">
         <v>10.93</v>
       </c>
-      <c r="J28" s="5">
+      <c r="J28" s="3">
         <v>140.05</v>
       </c>
-      <c r="K28" s="5">
+      <c r="K28" s="3">
         <v>1.24</v>
       </c>
-      <c r="L28" s="5">
+      <c r="L28" s="3">
         <v>4.24</v>
       </c>
-      <c r="M28" s="5">
+      <c r="M28" s="3">
         <v>0.392</v>
       </c>
-      <c r="N28" s="5">
+      <c r="N28" s="3">
         <v>14.11</v>
       </c>
-      <c r="O28" s="5">
+      <c r="O28" s="3">
         <v>20.8</v>
       </c>
-      <c r="P28" s="5">
+      <c r="P28" s="3">
         <v>1.234</v>
       </c>
-      <c r="Q28" s="5">
+      <c r="Q28" s="3">
         <v>2.69</v>
       </c>
-      <c r="R28" s="5">
+      <c r="R28" s="3">
         <v>2.6</v>
       </c>
-      <c r="S28" s="5">
+      <c r="S28" s="3">
         <v>2.18</v>
       </c>
-      <c r="T28" s="5">
+      <c r="T28" s="3">
         <v>51.98</v>
       </c>
-      <c r="U28" s="5">
+      <c r="U28" s="3">
         <v>7.5</v>
       </c>
-      <c r="V28" s="5">
+      <c r="V28" s="3">
         <v>0.42</v>
       </c>
-      <c r="W28" s="5">
+      <c r="W28" s="3">
         <v>100.9</v>
       </c>
     </row>
@@ -2600,70 +2588,70 @@
       <c r="A29" s="1" t="s">
         <v>52</v>
       </c>
-      <c r="B29" s="4">
+      <c r="B29" s="2">
         <v>473</v>
       </c>
-      <c r="C29" s="5">
+      <c r="C29" s="3">
         <v>0.442</v>
       </c>
-      <c r="D29" s="5">
+      <c r="D29" s="3">
         <v>1.04</v>
       </c>
-      <c r="E29" s="5">
+      <c r="E29" s="3">
         <v>0.4</v>
       </c>
-      <c r="F29" s="5">
+      <c r="F29" s="3">
         <v>3.61</v>
       </c>
-      <c r="G29" s="5">
+      <c r="G29" s="3">
         <v>67.2</v>
       </c>
-      <c r="H29" s="5">
+      <c r="H29" s="3">
         <v>5.66</v>
       </c>
-      <c r="I29" s="5">
+      <c r="I29" s="3">
         <v>20.43</v>
       </c>
-      <c r="J29" s="5">
+      <c r="J29" s="3">
         <v>944.61</v>
       </c>
-      <c r="K29" s="5">
+      <c r="K29" s="3">
         <v>7.99</v>
       </c>
-      <c r="L29" s="5">
+      <c r="L29" s="3">
         <v>0.66</v>
       </c>
-      <c r="M29" s="5">
+      <c r="M29" s="3">
         <v>0.523</v>
       </c>
-      <c r="N29" s="5">
+      <c r="N29" s="3">
         <v>10.82</v>
       </c>
-      <c r="O29" s="5">
+      <c r="O29" s="3">
         <v>18.6</v>
       </c>
-      <c r="P29" s="5">
+      <c r="P29" s="3">
         <v>1.265</v>
       </c>
-      <c r="Q29" s="5">
+      <c r="Q29" s="3">
         <v>2.72</v>
       </c>
-      <c r="R29" s="5">
+      <c r="R29" s="3">
         <v>2.63</v>
       </c>
-      <c r="S29" s="5">
+      <c r="S29" s="3">
         <v>0.34</v>
       </c>
-      <c r="T29" s="5">
+      <c r="T29" s="3">
         <v>346.66</v>
       </c>
-      <c r="U29" s="5">
+      <c r="U29" s="3">
         <v>6.53</v>
       </c>
-      <c r="V29" s="5">
+      <c r="V29" s="3">
         <v>0.78</v>
       </c>
-      <c r="W29" s="5">
+      <c r="W29" s="3">
         <v>13.9</v>
       </c>
     </row>
@@ -2671,70 +2659,70 @@
       <c r="A30" s="1" t="s">
         <v>53</v>
       </c>
-      <c r="B30" s="4">
+      <c r="B30" s="2">
         <v>298</v>
       </c>
-      <c r="C30" s="5">
+      <c r="C30" s="3">
         <v>0.463</v>
       </c>
-      <c r="D30" s="5">
+      <c r="D30" s="3">
         <v>1.13</v>
       </c>
-      <c r="E30" s="5">
+      <c r="E30" s="3">
         <v>0.45</v>
       </c>
-      <c r="F30" s="5">
+      <c r="F30" s="3">
         <v>3.17</v>
       </c>
-      <c r="G30" s="5">
+      <c r="G30" s="3">
         <v>53.7</v>
       </c>
-      <c r="H30" s="5">
+      <c r="H30" s="3">
         <v>5.7</v>
       </c>
-      <c r="I30" s="5">
+      <c r="I30" s="3">
         <v>18.1</v>
       </c>
-      <c r="J30" s="5">
+      <c r="J30" s="3">
         <v>710.1</v>
       </c>
-      <c r="K30" s="5">
+      <c r="K30" s="3">
         <v>7.09</v>
       </c>
-      <c r="L30" s="5">
+      <c r="L30" s="3">
         <v>0.96</v>
       </c>
-      <c r="M30" s="5">
+      <c r="M30" s="3">
         <v>0.649</v>
       </c>
-      <c r="N30" s="5">
+      <c r="N30" s="3">
         <v>8.79</v>
       </c>
-      <c r="O30" s="5">
+      <c r="O30" s="3">
         <v>16.9</v>
       </c>
-      <c r="P30" s="5">
+      <c r="P30" s="3">
         <v>1.276</v>
       </c>
-      <c r="Q30" s="5">
+      <c r="Q30" s="3">
         <v>2.74</v>
       </c>
-      <c r="R30" s="5">
+      <c r="R30" s="3">
         <v>2.64</v>
       </c>
-      <c r="S30" s="5">
+      <c r="S30" s="3">
         <v>0.39</v>
       </c>
-      <c r="T30" s="5">
+      <c r="T30" s="3">
         <v>259.56</v>
       </c>
-      <c r="U30" s="5">
+      <c r="U30" s="3">
         <v>4.11</v>
       </c>
-      <c r="V30" s="5">
+      <c r="V30" s="3">
         <v>0.69</v>
       </c>
-      <c r="W30" s="5">
+      <c r="W30" s="3">
         <v>12.8</v>
       </c>
     </row>
@@ -2742,70 +2730,70 @@
       <c r="A31" s="1" t="s">
         <v>54</v>
       </c>
-      <c r="B31" s="4">
+      <c r="B31" s="2">
         <v>548</v>
       </c>
-      <c r="C31" s="5">
+      <c r="C31" s="3">
         <v>0.845</v>
       </c>
-      <c r="D31" s="5">
+      <c r="D31" s="3">
         <v>0.989</v>
       </c>
-      <c r="E31" s="5">
+      <c r="E31" s="3">
         <v>3.88</v>
       </c>
-      <c r="F31" s="5">
+      <c r="F31" s="3">
         <v>1.99</v>
       </c>
-      <c r="G31" s="5">
+      <c r="G31" s="3">
         <v>31.3</v>
       </c>
-      <c r="H31" s="5">
+      <c r="H31" s="3">
         <v>7.5</v>
       </c>
-      <c r="I31" s="5">
+      <c r="I31" s="3">
         <v>14.91</v>
       </c>
-      <c r="J31" s="5">
+      <c r="J31" s="3">
         <v>263.15</v>
       </c>
-      <c r="K31" s="5">
+      <c r="K31" s="3">
         <v>1.37</v>
       </c>
-      <c r="L31" s="5">
+      <c r="L31" s="3">
         <v>2.26</v>
       </c>
-      <c r="M31" s="5">
+      <c r="M31" s="3">
         <v>1.698</v>
       </c>
-      <c r="N31" s="5">
+      <c r="N31" s="3">
         <v>4.42</v>
       </c>
-      <c r="O31" s="5">
+      <c r="O31" s="3">
         <v>15.8</v>
       </c>
-      <c r="P31" s="5">
+      <c r="P31" s="3">
         <v>1.646</v>
       </c>
-      <c r="Q31" s="5">
+      <c r="Q31" s="3">
         <v>3.14</v>
       </c>
-      <c r="R31" s="5">
+      <c r="R31" s="3">
         <v>3.03</v>
       </c>
-      <c r="S31" s="5">
+      <c r="S31" s="3">
         <v>2.29</v>
       </c>
-      <c r="T31" s="5">
+      <c r="T31" s="3">
         <v>83.82</v>
       </c>
-      <c r="U31" s="5">
+      <c r="U31" s="3">
         <v>7.57</v>
       </c>
-      <c r="V31" s="5">
+      <c r="V31" s="3">
         <v>0.49</v>
       </c>
-      <c r="W31" s="5">
+      <c r="W31" s="3">
         <v>63.4</v>
       </c>
     </row>
@@ -2813,70 +2801,70 @@
       <c r="A32" s="1" t="s">
         <v>55</v>
       </c>
-      <c r="B32" s="4">
+      <c r="B32" s="2">
         <v>463</v>
       </c>
-      <c r="C32" s="5">
+      <c r="C32" s="3">
         <v>1.03</v>
       </c>
-      <c r="D32" s="5">
+      <c r="D32" s="3">
         <v>0.766</v>
       </c>
-      <c r="E32" s="5">
+      <c r="E32" s="3">
         <v>1.69</v>
       </c>
-      <c r="F32" s="5">
+      <c r="F32" s="3">
         <v>2.1</v>
       </c>
-      <c r="G32" s="5">
+      <c r="G32" s="3">
         <v>42.4</v>
       </c>
-      <c r="H32" s="5">
+      <c r="H32" s="3">
         <v>7.99</v>
       </c>
-      <c r="I32" s="5">
+      <c r="I32" s="3">
         <v>16.9</v>
       </c>
-      <c r="J32" s="5">
+      <c r="J32" s="3">
         <v>278.7</v>
       </c>
-      <c r="K32" s="5">
+      <c r="K32" s="3">
         <v>6.62</v>
       </c>
-      <c r="L32" s="5">
+      <c r="L32" s="3">
         <v>1.66</v>
       </c>
-      <c r="M32" s="5">
+      <c r="M32" s="3">
         <v>1.274</v>
       </c>
-      <c r="N32" s="5">
+      <c r="N32" s="3">
         <v>6.27</v>
       </c>
-      <c r="O32" s="5">
+      <c r="O32" s="3">
         <v>20.2</v>
       </c>
-      <c r="P32" s="5">
+      <c r="P32" s="3">
         <v>1.728</v>
       </c>
-      <c r="Q32" s="5">
+      <c r="Q32" s="3">
         <v>3.24</v>
       </c>
-      <c r="R32" s="5">
+      <c r="R32" s="3">
         <v>3.12</v>
       </c>
-      <c r="S32" s="5">
+      <c r="S32" s="3">
         <v>0.49</v>
       </c>
-      <c r="T32" s="5">
+      <c r="T32" s="3">
         <v>86.03</v>
       </c>
-      <c r="U32" s="5">
+      <c r="U32" s="3">
         <v>6.39</v>
       </c>
-      <c r="V32" s="5">
+      <c r="V32" s="3">
         <v>0.54</v>
       </c>
-      <c r="W32" s="5">
+      <c r="W32" s="3">
         <v>40.5</v>
       </c>
     </row>
@@ -2884,70 +2872,70 @@
       <c r="A33" s="1" t="s">
         <v>56</v>
       </c>
-      <c r="B33" s="4">
+      <c r="B33" s="2">
         <v>413</v>
       </c>
-      <c r="C33" s="5">
+      <c r="C33" s="3">
         <v>1.25</v>
       </c>
-      <c r="D33" s="5">
+      <c r="D33" s="3">
         <v>0.785</v>
       </c>
-      <c r="E33" s="5">
+      <c r="E33" s="3">
         <v>3.25</v>
       </c>
-      <c r="F33" s="5">
+      <c r="F33" s="3">
         <v>1.69</v>
       </c>
-      <c r="G33" s="5">
+      <c r="G33" s="3">
         <v>32.2</v>
       </c>
-      <c r="H33" s="5">
+      <c r="H33" s="3">
         <v>8.09</v>
       </c>
-      <c r="I33" s="5">
+      <c r="I33" s="3">
         <v>13.7</v>
       </c>
-      <c r="J33" s="5">
+      <c r="J33" s="3">
         <v>150.4</v>
       </c>
-      <c r="K33" s="5">
+      <c r="K33" s="3">
         <v>5.36</v>
       </c>
-      <c r="L33" s="5">
+      <c r="L33" s="3">
         <v>3.14</v>
       </c>
-      <c r="M33" s="5">
+      <c r="M33" s="3">
         <v>1.466</v>
       </c>
-      <c r="N33" s="5">
+      <c r="N33" s="3">
         <v>5.52</v>
       </c>
-      <c r="O33" s="4">
+      <c r="O33" s="2">
         <v>19</v>
       </c>
-      <c r="P33" s="5">
+      <c r="P33" s="3">
         <v>1.744</v>
       </c>
-      <c r="Q33" s="5">
+      <c r="Q33" s="3">
         <v>3.26</v>
       </c>
-      <c r="R33" s="5">
+      <c r="R33" s="3">
         <v>3.14</v>
       </c>
-      <c r="S33" s="5">
+      <c r="S33" s="3">
         <v>0.61</v>
       </c>
-      <c r="T33" s="5">
+      <c r="T33" s="3">
         <v>46.15</v>
       </c>
-      <c r="U33" s="5">
+      <c r="U33" s="3">
         <v>5.7</v>
       </c>
-      <c r="V33" s="5">
+      <c r="V33" s="3">
         <v>0.44</v>
       </c>
-      <c r="W33" s="4">
+      <c r="W33" s="2">
         <v>69</v>
       </c>
     </row>
@@ -2955,70 +2943,70 @@
       <c r="A34" s="1" t="s">
         <v>57</v>
       </c>
-      <c r="B34" s="4">
+      <c r="B34" s="2">
         <v>298</v>
       </c>
-      <c r="C34" s="5">
+      <c r="C34" s="3">
         <v>0.442</v>
       </c>
-      <c r="D34" s="5">
+      <c r="D34" s="3">
         <v>0.98</v>
       </c>
-      <c r="E34" s="5">
+      <c r="E34" s="3">
         <v>0.2</v>
       </c>
-      <c r="F34" s="5">
+      <c r="F34" s="3">
         <v>3.83</v>
       </c>
-      <c r="G34" s="5">
+      <c r="G34" s="3">
         <v>73.3</v>
       </c>
-      <c r="H34" s="5">
+      <c r="H34" s="3">
         <v>8.34</v>
       </c>
-      <c r="I34" s="5">
+      <c r="I34" s="3">
         <v>31.9</v>
       </c>
-      <c r="J34" s="4">
+      <c r="J34" s="2">
         <v>2295</v>
       </c>
-      <c r="K34" s="5">
+      <c r="K34" s="3">
         <v>12.45</v>
       </c>
-      <c r="L34" s="5">
+      <c r="L34" s="3">
         <v>0.26</v>
       </c>
-      <c r="M34" s="5">
+      <c r="M34" s="3">
         <v>1.578</v>
       </c>
-      <c r="N34" s="5">
+      <c r="N34" s="3">
         <v>5.29</v>
       </c>
-      <c r="O34" s="5">
+      <c r="O34" s="3">
         <v>19.1</v>
       </c>
-      <c r="P34" s="5">
+      <c r="P34" s="3">
         <v>1.785</v>
       </c>
-      <c r="Q34" s="5">
+      <c r="Q34" s="3">
         <v>3.31</v>
       </c>
-      <c r="R34" s="5">
+      <c r="R34" s="3">
         <v>3.19</v>
       </c>
-      <c r="S34" s="5">
+      <c r="S34" s="3">
         <v>0.27</v>
       </c>
-      <c r="T34" s="5">
+      <c r="T34" s="3">
         <v>693.22</v>
       </c>
-      <c r="U34" s="5">
+      <c r="U34" s="3">
         <v>4.11</v>
       </c>
-      <c r="V34" s="4">
+      <c r="V34" s="2">
         <v>1</v>
       </c>
-      <c r="W34" s="5">
+      <c r="W34" s="3">
         <v>4.1</v>
       </c>
     </row>
@@ -3026,70 +3014,70 @@
       <c r="A35" s="1" t="s">
         <v>58</v>
       </c>
-      <c r="B35" s="4">
+      <c r="B35" s="2">
         <v>473</v>
       </c>
-      <c r="C35" s="5">
+      <c r="C35" s="3">
         <v>0.864</v>
       </c>
-      <c r="D35" s="5">
+      <c r="D35" s="3">
         <v>1.14</v>
       </c>
-      <c r="E35" s="5">
+      <c r="E35" s="3">
         <v>3.38</v>
       </c>
-      <c r="F35" s="5">
+      <c r="F35" s="3">
         <v>1.69</v>
       </c>
-      <c r="G35" s="5">
+      <c r="G35" s="3">
         <v>33.9</v>
       </c>
-      <c r="H35" s="5">
+      <c r="H35" s="3">
         <v>10.93</v>
       </c>
-      <c r="I35" s="5">
+      <c r="I35" s="3">
         <v>18.43</v>
       </c>
-      <c r="J35" s="5">
+      <c r="J35" s="3">
         <v>393.25</v>
       </c>
-      <c r="K35" s="5">
+      <c r="K35" s="3">
         <v>1.55</v>
       </c>
-      <c r="L35" s="5">
+      <c r="L35" s="3">
         <v>1.75</v>
       </c>
-      <c r="M35" s="5">
+      <c r="M35" s="3">
         <v>3.237</v>
       </c>
-      <c r="N35" s="5">
+      <c r="N35" s="3">
         <v>3.38</v>
       </c>
-      <c r="O35" s="5">
+      <c r="O35" s="3">
         <v>20.1</v>
       </c>
-      <c r="P35" s="5">
+      <c r="P35" s="3">
         <v>2.136</v>
       </c>
-      <c r="Q35" s="5">
+      <c r="Q35" s="3">
         <v>3.79</v>
       </c>
-      <c r="R35" s="5">
+      <c r="R35" s="3">
         <v>3.65</v>
       </c>
-      <c r="S35" s="5">
+      <c r="S35" s="3">
         <v>2.45</v>
       </c>
-      <c r="T35" s="5">
+      <c r="T35" s="3">
         <v>103.76</v>
       </c>
-      <c r="U35" s="5">
+      <c r="U35" s="3">
         <v>6.53</v>
       </c>
-      <c r="V35" s="5">
+      <c r="V35" s="3">
         <v>0.5</v>
       </c>
-      <c r="W35" s="4">
+      <c r="W35" s="2">
         <v>51</v>
       </c>
     </row>
@@ -3097,70 +3085,70 @@
       <c r="A36" s="1" t="s">
         <v>59</v>
       </c>
-      <c r="B36" s="4">
+      <c r="B36" s="2">
         <v>298</v>
       </c>
-      <c r="C36" s="5">
+      <c r="C36" s="3">
         <v>1.4</v>
       </c>
-      <c r="D36" s="5">
+      <c r="D36" s="3">
         <v>0.851</v>
       </c>
-      <c r="E36" s="5">
+      <c r="E36" s="3">
         <v>4.38</v>
       </c>
-      <c r="F36" s="5">
+      <c r="F36" s="3">
         <v>1.39</v>
       </c>
-      <c r="G36" s="4">
+      <c r="G36" s="2">
         <v>26</v>
       </c>
-      <c r="H36" s="5">
+      <c r="H36" s="3">
         <v>11.1</v>
       </c>
-      <c r="I36" s="5">
+      <c r="I36" s="3">
         <v>15.4</v>
       </c>
-      <c r="J36" s="5">
+      <c r="J36" s="3">
         <v>168.3</v>
       </c>
-      <c r="K36" s="4">
+      <c r="K36" s="2">
         <v>6</v>
       </c>
-      <c r="L36" s="5">
+      <c r="L36" s="3">
         <v>3.04</v>
       </c>
-      <c r="M36" s="5">
+      <c r="M36" s="3">
         <v>3.884</v>
       </c>
-      <c r="N36" s="5">
+      <c r="N36" s="3">
         <v>2.86</v>
       </c>
-      <c r="O36" s="5">
+      <c r="O36" s="3">
         <v>18.6</v>
       </c>
-      <c r="P36" s="5">
+      <c r="P36" s="3">
         <v>2.156</v>
       </c>
-      <c r="Q36" s="5">
+      <c r="Q36" s="3">
         <v>3.82</v>
       </c>
-      <c r="R36" s="5">
+      <c r="R36" s="3">
         <v>3.68</v>
       </c>
-      <c r="S36" s="5">
+      <c r="S36" s="3">
         <v>0.64</v>
       </c>
-      <c r="T36" s="5">
+      <c r="T36" s="3">
         <v>44.07</v>
       </c>
-      <c r="U36" s="5">
+      <c r="U36" s="3">
         <v>4.11</v>
       </c>
-      <c r="V36" s="5">
+      <c r="V36" s="3">
         <v>0.42</v>
       </c>
-      <c r="W36" s="5">
+      <c r="W36" s="3">
         <v>56.4</v>
       </c>
     </row>
@@ -3168,70 +3156,70 @@
       <c r="A37" s="1" t="s">
         <v>60</v>
       </c>
-      <c r="B37" s="4">
+      <c r="B37" s="2">
         <v>653</v>
       </c>
-      <c r="C37" s="5">
+      <c r="C37" s="3">
         <v>0.598</v>
       </c>
-      <c r="D37" s="5">
+      <c r="D37" s="3">
         <v>1.46</v>
       </c>
-      <c r="E37" s="5">
+      <c r="E37" s="3">
         <v>2.12</v>
       </c>
-      <c r="F37" s="5">
+      <c r="F37" s="3">
         <v>1.9</v>
       </c>
-      <c r="G37" s="5">
+      <c r="G37" s="3">
         <v>47.2</v>
       </c>
-      <c r="H37" s="5">
+      <c r="H37" s="3">
         <v>12.3</v>
       </c>
-      <c r="I37" s="5">
+      <c r="I37" s="3">
         <v>23.4</v>
       </c>
-      <c r="J37" s="5">
+      <c r="J37" s="3">
         <v>915.41</v>
       </c>
-      <c r="K37" s="5">
+      <c r="K37" s="3">
         <v>9.15</v>
       </c>
-      <c r="L37" s="5">
+      <c r="L37" s="3">
         <v>0.96</v>
       </c>
-      <c r="M37" s="5">
+      <c r="M37" s="3">
         <v>3.019</v>
       </c>
-      <c r="N37" s="5">
+      <c r="N37" s="3">
         <v>4.07</v>
       </c>
-      <c r="O37" s="5">
+      <c r="O37" s="3">
         <v>24.8</v>
       </c>
-      <c r="P37" s="5">
+      <c r="P37" s="3">
         <v>2.291</v>
       </c>
-      <c r="Q37" s="5">
+      <c r="Q37" s="3">
         <v>4.02</v>
       </c>
-      <c r="R37" s="5">
+      <c r="R37" s="3">
         <v>3.87</v>
       </c>
-      <c r="S37" s="5">
+      <c r="S37" s="3">
         <v>0.44</v>
       </c>
-      <c r="T37" s="5">
+      <c r="T37" s="3">
         <v>227.7</v>
       </c>
-      <c r="U37" s="5">
+      <c r="U37" s="3">
         <v>9.02</v>
       </c>
-      <c r="V37" s="5">
+      <c r="V37" s="3">
         <v>0.6</v>
       </c>
-      <c r="W37" s="5">
+      <c r="W37" s="3">
         <v>41.1</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Incorporated the characteristic ratio as an additional polymer property in the everaers_et_al_unit_properties JSON and Excel files, and incorporated the characteristic ratio as a required parameter in the bead_spring_parameter_provider Python file. Finally, a typo in calculating the box volume was corrected in several network generator example Python files.
</commit_message>
<xml_diff>
--- a/src/pylimer_tools/data/everaers_et_al_unit_properties.xlsx
+++ b/src/pylimer_tools/data/everaers_et_al_unit_properties.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="10315"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="11102"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/timbernhard/Privat/Programming/OpenSource-Contributions/pylimer-tools/src/pylimer_tools/data/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jasonmulderrig/research/projects/polydisperse-polymer-networks/lib/python3.12/site-packages/pylimer_tools/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2FFC8C68-1CFD-A147-8F24-B65093CCF391}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EE60E0D8-FEC9-3347-A01F-59A61E7488B3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="760" windowWidth="34560" windowHeight="21580" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="720" windowWidth="29400" windowHeight="18400" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="60" uniqueCount="60">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="61" uniqueCount="61">
   <si>
     <t>name</t>
   </si>
@@ -112,9 +112,6 @@
     <t>PIB(413)</t>
   </si>
   <si>
-    <t>cis-P1</t>
-  </si>
-  <si>
     <t>a-PP(463)</t>
   </si>
   <si>
@@ -200,13 +197,19 @@
   </si>
   <si>
     <t>PTFE*</t>
+  </si>
+  <si>
+    <t>C_inf</t>
+  </si>
+  <si>
+    <t>cis-PI</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -219,6 +222,12 @@
       <color rgb="FF000000"/>
       <name val="Calibri"/>
       <family val="2"/>
+    </font>
+    <font>
+      <sz val="8"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
@@ -269,7 +278,7 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="24">
+  <dxfs count="25">
     <dxf>
       <font>
         <b val="0"/>
@@ -727,7 +736,7 @@
         <family val="2"/>
         <scheme val="none"/>
       </font>
-      <numFmt numFmtId="4" formatCode="#,##0.00"/>
+      <numFmt numFmtId="2" formatCode="0.00"/>
       <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
@@ -749,6 +758,26 @@
       </font>
       <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <numFmt numFmtId="4" formatCode="#,##0.00"/>
+      <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
@@ -763,32 +792,33 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{87C85193-D6C5-4C49-B027-4C18B1B0E045}" name="Table1" displayName="Table1" ref="A1:W37" totalsRowShown="0" headerRowDxfId="22" dataDxfId="23">
-  <autoFilter ref="A1:W37" xr:uid="{87C85193-D6C5-4C49-B027-4C18B1B0E045}"/>
-  <tableColumns count="23">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{87C85193-D6C5-4C49-B027-4C18B1B0E045}" name="Table1" displayName="Table1" ref="A1:X37" totalsRowShown="0" headerRowDxfId="24" dataDxfId="23">
+  <autoFilter ref="A1:X37" xr:uid="{87C85193-D6C5-4C49-B027-4C18B1B0E045}"/>
+  <tableColumns count="24">
     <tableColumn id="1" xr3:uid="{09978F38-00B1-454F-B36F-ED2DD365FFB9}" name="name"/>
-    <tableColumn id="2" xr3:uid="{0E5252E0-ECE6-0949-95DC-DD29C8CFFF07}" name="T_ref" dataDxfId="21"/>
-    <tableColumn id="3" xr3:uid="{5FC94EDA-4E44-A345-B564-14BE5DA189C7}" name="R_to_2_over_M_c" dataDxfId="20"/>
-    <tableColumn id="4" xr3:uid="{FF1E1487-BD89-874E-B0BA-427CD1837CBA}" name="rho_bulk" dataDxfId="19"/>
-    <tableColumn id="5" xr3:uid="{AB726438-CCD6-9849-ADC3-EB349EDFBC0B}" name="G_e" dataDxfId="18"/>
-    <tableColumn id="6" xr3:uid="{F3637338-6243-6E4E-95AB-04BA90F0DC13}" name="p" dataDxfId="17"/>
-    <tableColumn id="7" xr3:uid="{457612CA-7A7C-2B47-B2C9-5C601A0E2F1F}" name="d_T" dataDxfId="16"/>
-    <tableColumn id="8" xr3:uid="{38312A95-9D55-9B41-980E-AC4D1DA1075B}" name="n_K" dataDxfId="15"/>
-    <tableColumn id="9" xr3:uid="{C017CDE7-FD43-144E-A9B7-36FB7552AE70}" name="l_K" dataDxfId="14"/>
-    <tableColumn id="10" xr3:uid="{C1A05868-8FC2-D645-81EC-68F176BAC4A9}" name="M_k" dataDxfId="13"/>
-    <tableColumn id="11" xr3:uid="{2C3CCC47-CC8C-5C48-87F8-4F1B1D9FAEBB}" name="M_k_over_M_m" dataDxfId="12"/>
-    <tableColumn id="12" xr3:uid="{140DD038-1AC8-D64A-81D4-45A3588748A2}" name="rho_K" dataDxfId="11"/>
-    <tableColumn id="13" xr3:uid="{534D6626-9284-EA4C-A4FB-9BAD1198E8CB}" name="G_e_times_l_K_to_3" dataDxfId="10"/>
-    <tableColumn id="14" xr3:uid="{3EAD4852-3AF4-DA46-BFA4-DF6C2FC535F8}" name="N_ek" dataDxfId="9"/>
-    <tableColumn id="15" xr3:uid="{59F85AC7-BD45-0C4C-B003-7D1274E1C189}" name="alpha" dataDxfId="8"/>
-    <tableColumn id="16" xr3:uid="{3F8D6442-276F-7141-A167-C37C2F9AC155}" name="kappa" dataDxfId="7"/>
-    <tableColumn id="17" xr3:uid="{5E0DA02E-9669-E44D-8613-D84EFC63C613}" name="Cb" dataDxfId="6"/>
-    <tableColumn id="18" xr3:uid="{CDA5AED2-3254-C846-844E-983C0EB17D56}" name="l_k_over_sigma" dataDxfId="5"/>
-    <tableColumn id="19" xr3:uid="{CD8F483D-8D87-1C4E-A33C-8373F7D627DB}" name="Mm_over_Mb" dataDxfId="4"/>
-    <tableColumn id="20" xr3:uid="{2534DDBF-0A92-D444-A414-140F02A2B0D3}" name="Mb" dataDxfId="3"/>
-    <tableColumn id="21" xr3:uid="{05FB0CA7-5AA9-264D-B34A-CDE4B3331BF2}" name="kB_Tref" dataDxfId="2"/>
-    <tableColumn id="22" xr3:uid="{6C2D3A19-BAE0-4D4C-8A43-DBDFC6EC864B}" name="sigma" dataDxfId="1"/>
-    <tableColumn id="23" xr3:uid="{240EEFC7-5DDC-7E49-A72C-D40F2E2B66E3}" name="kB_Tref_over_sigma_to_3" dataDxfId="0"/>
+    <tableColumn id="2" xr3:uid="{0E5252E0-ECE6-0949-95DC-DD29C8CFFF07}" name="T_ref" dataDxfId="22"/>
+    <tableColumn id="3" xr3:uid="{5FC94EDA-4E44-A345-B564-14BE5DA189C7}" name="R_to_2_over_M_c" dataDxfId="21"/>
+    <tableColumn id="4" xr3:uid="{FF1E1487-BD89-874E-B0BA-427CD1837CBA}" name="rho_bulk" dataDxfId="20"/>
+    <tableColumn id="5" xr3:uid="{AB726438-CCD6-9849-ADC3-EB349EDFBC0B}" name="G_e" dataDxfId="19"/>
+    <tableColumn id="6" xr3:uid="{F3637338-6243-6E4E-95AB-04BA90F0DC13}" name="p" dataDxfId="18"/>
+    <tableColumn id="7" xr3:uid="{457612CA-7A7C-2B47-B2C9-5C601A0E2F1F}" name="d_T" dataDxfId="17"/>
+    <tableColumn id="8" xr3:uid="{38312A95-9D55-9B41-980E-AC4D1DA1075B}" name="n_K" dataDxfId="16"/>
+    <tableColumn id="9" xr3:uid="{C017CDE7-FD43-144E-A9B7-36FB7552AE70}" name="l_K" dataDxfId="15"/>
+    <tableColumn id="10" xr3:uid="{C1A05868-8FC2-D645-81EC-68F176BAC4A9}" name="M_k" dataDxfId="14"/>
+    <tableColumn id="11" xr3:uid="{2C3CCC47-CC8C-5C48-87F8-4F1B1D9FAEBB}" name="M_k_over_M_m" dataDxfId="13"/>
+    <tableColumn id="12" xr3:uid="{140DD038-1AC8-D64A-81D4-45A3588748A2}" name="rho_K" dataDxfId="12"/>
+    <tableColumn id="13" xr3:uid="{534D6626-9284-EA4C-A4FB-9BAD1198E8CB}" name="G_e_times_l_K_to_3" dataDxfId="11"/>
+    <tableColumn id="14" xr3:uid="{3EAD4852-3AF4-DA46-BFA4-DF6C2FC535F8}" name="N_ek" dataDxfId="10"/>
+    <tableColumn id="15" xr3:uid="{59F85AC7-BD45-0C4C-B003-7D1274E1C189}" name="alpha" dataDxfId="9"/>
+    <tableColumn id="16" xr3:uid="{3F8D6442-276F-7141-A167-C37C2F9AC155}" name="kappa" dataDxfId="8"/>
+    <tableColumn id="17" xr3:uid="{5E0DA02E-9669-E44D-8613-D84EFC63C613}" name="Cb" dataDxfId="7"/>
+    <tableColumn id="18" xr3:uid="{CDA5AED2-3254-C846-844E-983C0EB17D56}" name="l_k_over_sigma" dataDxfId="6"/>
+    <tableColumn id="19" xr3:uid="{CD8F483D-8D87-1C4E-A33C-8373F7D627DB}" name="Mm_over_Mb" dataDxfId="5"/>
+    <tableColumn id="20" xr3:uid="{2534DDBF-0A92-D444-A414-140F02A2B0D3}" name="Mb" dataDxfId="4"/>
+    <tableColumn id="21" xr3:uid="{05FB0CA7-5AA9-264D-B34A-CDE4B3331BF2}" name="kB_Tref" dataDxfId="3"/>
+    <tableColumn id="22" xr3:uid="{6C2D3A19-BAE0-4D4C-8A43-DBDFC6EC864B}" name="sigma" dataDxfId="2"/>
+    <tableColumn id="23" xr3:uid="{240EEFC7-5DDC-7E49-A72C-D40F2E2B66E3}" name="kB_Tref_over_sigma_to_3" dataDxfId="1"/>
+    <tableColumn id="24" xr3:uid="{5A986246-C3BC-2E43-9972-4DD318FEA984}" name="C_inf" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1082,7 +1112,7 @@
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
-  <dimension ref="A1:W37"/>
+  <dimension ref="A1:X37"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="13" bestFit="1" customWidth="1"/>
@@ -1101,7 +1131,7 @@
     <col min="23" max="23" width="22.6640625" style="4" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:23" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:24" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1171,8 +1201,11 @@
       <c r="W1" s="2" t="s">
         <v>22</v>
       </c>
+      <c r="X1" s="2" t="s">
+        <v>59</v>
+      </c>
     </row>
-    <row r="2" spans="1:23" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:24" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>23</v>
       </c>
@@ -1242,8 +1275,11 @@
       <c r="W2" s="5">
         <v>32</v>
       </c>
+      <c r="X2" s="5">
+        <v>4.8</v>
+      </c>
     </row>
-    <row r="3" spans="1:23" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:24" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>24</v>
       </c>
@@ -1313,8 +1349,11 @@
       <c r="W3" s="5">
         <v>41.3</v>
       </c>
+      <c r="X3" s="5">
+        <v>4.7</v>
+      </c>
     </row>
-    <row r="4" spans="1:23" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:24" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>25</v>
       </c>
@@ -1384,8 +1423,11 @@
       <c r="W4" s="5">
         <v>17.600000000000001</v>
       </c>
+      <c r="X4" s="5">
+        <v>5.78</v>
+      </c>
     </row>
-    <row r="5" spans="1:23" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:24" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>26</v>
       </c>
@@ -1455,8 +1497,11 @@
       <c r="W5" s="5">
         <v>37.1</v>
       </c>
+      <c r="X5" s="5">
+        <v>4.96</v>
+      </c>
     </row>
-    <row r="6" spans="1:23" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:24" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>27</v>
       </c>
@@ -1526,8 +1571,11 @@
       <c r="W6" s="5">
         <v>33.1</v>
       </c>
+      <c r="X6" s="5">
+        <v>5.26</v>
+      </c>
     </row>
-    <row r="7" spans="1:23" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:24" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>28</v>
       </c>
@@ -1597,8 +1645,11 @@
       <c r="W7" s="5">
         <v>61.3</v>
       </c>
+      <c r="X7" s="5">
+        <v>4.6100000000000003</v>
+      </c>
     </row>
-    <row r="8" spans="1:23" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:24" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
         <v>29</v>
       </c>
@@ -1668,10 +1719,13 @@
       <c r="W8" s="5">
         <v>27.3</v>
       </c>
+      <c r="X8" s="5">
+        <v>6.58</v>
+      </c>
     </row>
-    <row r="9" spans="1:23" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:24" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
-        <v>30</v>
+        <v>60</v>
       </c>
       <c r="B9" s="5">
         <v>298</v>
@@ -1739,10 +1793,13 @@
       <c r="W9" s="5">
         <v>44</v>
       </c>
+      <c r="X9" s="5">
+        <v>5.2</v>
+      </c>
     </row>
-    <row r="10" spans="1:23" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:24" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B10" s="5">
         <v>463</v>
@@ -1810,10 +1867,13 @@
       <c r="W10" s="5">
         <v>40.700000000000003</v>
       </c>
+      <c r="X10" s="5">
+        <v>6</v>
+      </c>
     </row>
-    <row r="11" spans="1:23" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:24" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B11" s="5">
         <v>463</v>
@@ -1881,10 +1941,13 @@
       <c r="W11" s="5">
         <v>40.4</v>
       </c>
+      <c r="X11" s="5">
+        <v>6.15</v>
+      </c>
     </row>
-    <row r="12" spans="1:23" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:24" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B12" s="5">
         <v>413</v>
@@ -1952,10 +2015,13 @@
       <c r="W12" s="5">
         <v>38.200000000000003</v>
       </c>
+      <c r="X12" s="5">
+        <v>6</v>
+      </c>
     </row>
-    <row r="13" spans="1:23" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:24" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="B13" s="5">
         <v>348</v>
@@ -2023,10 +2089,13 @@
       <c r="W13" s="5">
         <v>34.299999999999997</v>
       </c>
+      <c r="X13" s="5">
+        <v>6</v>
+      </c>
     </row>
-    <row r="14" spans="1:23" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:24" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="B14" s="5">
         <v>298</v>
@@ -2094,10 +2163,13 @@
       <c r="W14" s="5">
         <v>30.7</v>
       </c>
+      <c r="X14" s="5">
+        <v>6</v>
+      </c>
     </row>
-    <row r="15" spans="1:23" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:24" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="B15" s="5">
         <v>298</v>
@@ -2165,10 +2237,13 @@
       <c r="W15" s="5">
         <v>22.2</v>
       </c>
+      <c r="X15" s="5">
+        <v>6.73</v>
+      </c>
     </row>
-    <row r="16" spans="1:23" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:24" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="B16" s="5">
         <v>413</v>
@@ -2236,10 +2311,13 @@
       <c r="W16" s="5">
         <v>17.600000000000001</v>
       </c>
+      <c r="X16" s="5">
+        <v>8.2200000000000006</v>
+      </c>
     </row>
-    <row r="17" spans="1:23" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:24" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="B17" s="5">
         <v>413</v>
@@ -2307,10 +2385,13 @@
       <c r="W17" s="5">
         <v>13.2</v>
       </c>
+      <c r="X17" s="5">
+        <v>9.34</v>
+      </c>
     </row>
-    <row r="18" spans="1:23" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:24" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B18" s="5">
         <v>298</v>
@@ -2378,10 +2459,13 @@
       <c r="W18" s="5">
         <v>15.6</v>
       </c>
+      <c r="X18" s="5">
+        <v>7.91</v>
+      </c>
     </row>
-    <row r="19" spans="1:23" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:24" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="B19" s="5">
         <v>298</v>
@@ -2449,10 +2533,13 @@
       <c r="W19" s="5">
         <v>15.9</v>
       </c>
+      <c r="X19" s="5">
+        <v>8.07</v>
+      </c>
     </row>
-    <row r="20" spans="1:23" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:24" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B20" s="5">
         <v>298</v>
@@ -2520,10 +2607,13 @@
       <c r="W20" s="5">
         <v>52.2</v>
       </c>
+      <c r="X20" s="5">
+        <v>5.61</v>
+      </c>
     </row>
-    <row r="21" spans="1:23" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:24" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="B21" s="5">
         <v>413</v>
@@ -2591,10 +2681,13 @@
       <c r="W21" s="5">
         <v>13.2</v>
       </c>
+      <c r="X21" s="5">
+        <v>9.7200000000000006</v>
+      </c>
     </row>
-    <row r="22" spans="1:23" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:24" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="B22" s="5">
         <v>300</v>
@@ -2662,10 +2755,13 @@
       <c r="W22" s="5">
         <v>23.1</v>
       </c>
+      <c r="X22" s="5">
+        <v>7.39</v>
+      </c>
     </row>
-    <row r="23" spans="1:23" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:24" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="B23" s="5">
         <v>353</v>
@@ -2698,7 +2794,7 @@
         <v>2.66</v>
       </c>
       <c r="L23" s="5" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="M23" s="5">
         <v>0.42299999999999999</v>
@@ -2733,10 +2829,13 @@
       <c r="W23" s="5">
         <v>80.2</v>
       </c>
+      <c r="X23" s="5">
+        <v>5.51</v>
+      </c>
     </row>
-    <row r="24" spans="1:23" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:24" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="B24" s="5">
         <v>473</v>
@@ -2804,10 +2903,13 @@
       <c r="W24" s="5">
         <v>111.5</v>
       </c>
+      <c r="X24" s="5">
+        <v>5.59</v>
+      </c>
     </row>
-    <row r="25" spans="1:23" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:24" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="B25" s="5">
         <v>373</v>
@@ -2875,10 +2977,13 @@
       <c r="W25" s="5">
         <v>5.7</v>
       </c>
+      <c r="X25" s="5">
+        <v>13.1</v>
+      </c>
     </row>
-    <row r="26" spans="1:23" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:24" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A26" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B26" s="5">
         <v>333</v>
@@ -2946,10 +3051,13 @@
       <c r="W26" s="5">
         <v>16.7</v>
       </c>
+      <c r="X26" s="5">
+        <v>4.6100000000000003</v>
+      </c>
     </row>
-    <row r="27" spans="1:23" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:24" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A27" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="B27" s="5">
         <v>298</v>
@@ -3017,10 +3125,13 @@
       <c r="W27" s="5">
         <v>40.6</v>
       </c>
+      <c r="X27" s="5">
+        <v>6.41</v>
+      </c>
     </row>
-    <row r="28" spans="1:23" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:24" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A28" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="B28" s="5">
         <v>543</v>
@@ -3088,10 +3199,13 @@
       <c r="W28" s="5">
         <v>100.9</v>
       </c>
+      <c r="X28" s="5">
+        <v>6.02</v>
+      </c>
     </row>
-    <row r="29" spans="1:23" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:24" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A29" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="B29" s="5">
         <v>473</v>
@@ -3159,10 +3273,13 @@
       <c r="W29" s="5">
         <v>13.9</v>
       </c>
+      <c r="X29" s="5">
+        <v>7.44</v>
+      </c>
     </row>
-    <row r="30" spans="1:23" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:24" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A30" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="B30" s="5">
         <v>298</v>
@@ -3230,10 +3347,13 @@
       <c r="W30" s="5">
         <v>12.8</v>
       </c>
+      <c r="X30" s="5">
+        <v>9.76</v>
+      </c>
     </row>
-    <row r="31" spans="1:23" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:24" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A31" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="B31" s="5">
         <v>548</v>
@@ -3301,10 +3421,13 @@
       <c r="W31" s="5">
         <v>63.4</v>
       </c>
+      <c r="X31" s="5">
+        <v>7.63</v>
+      </c>
     </row>
-    <row r="32" spans="1:23" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:24" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A32" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B32" s="5">
         <v>463</v>
@@ -3372,10 +3495,13 @@
       <c r="W32" s="5">
         <v>40.5</v>
       </c>
+      <c r="X32" s="5">
+        <v>9.1199999999999992</v>
+      </c>
     </row>
-    <row r="33" spans="1:23" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:24" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A33" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="B33" s="5">
         <v>413</v>
@@ -3443,10 +3569,13 @@
       <c r="W33" s="5">
         <v>69</v>
       </c>
+      <c r="X33" s="5">
+        <v>7.38</v>
+      </c>
     </row>
-    <row r="34" spans="1:23" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="34" spans="1:24" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A34" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="B34" s="5">
         <v>298</v>
@@ -3514,10 +3643,13 @@
       <c r="W34" s="5">
         <v>4.0999999999999996</v>
       </c>
+      <c r="X34" s="5">
+        <v>17.100000000000001</v>
+      </c>
     </row>
-    <row r="35" spans="1:23" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:24" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A35" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="B35" s="5">
         <v>473</v>
@@ -3585,10 +3717,13 @@
       <c r="W35" s="5">
         <v>51</v>
       </c>
+      <c r="X35" s="5">
+        <v>7.81</v>
+      </c>
     </row>
-    <row r="36" spans="1:23" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="36" spans="1:24" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A36" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B36" s="5">
         <v>298</v>
@@ -3656,10 +3791,13 @@
       <c r="W36" s="5">
         <v>56.4</v>
       </c>
+      <c r="X36" s="5">
+        <v>8.26</v>
+      </c>
     </row>
-    <row r="37" spans="1:23" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="37" spans="1:24" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A37" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="B37" s="5">
         <v>653</v>
@@ -3727,8 +3865,12 @@
       <c r="W37" s="5">
         <v>41.1</v>
       </c>
+      <c r="X37" s="5">
+        <v>12.78</v>
+      </c>
     </row>
   </sheetData>
+  <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">
     <tablePart r:id="rId1"/>

</xml_diff>